<commit_message>
ci: separate workflows for Appium, Selenium and Vulnerability scanning
</commit_message>
<xml_diff>
--- a/automation/excel/Mobile_E2E_Report_300_Passed.xlsx
+++ b/automation/excel/Mobile_E2E_Report_300_Passed.xlsx
@@ -33,7 +33,7 @@
     <t>Execution Timestamp</t>
   </si>
   <si>
-    <t>Tue, 21 Jul 2026 03:10:41 GMT</t>
+    <t>Wed, 22 Jul 2026 04:49:50 GMT</t>
   </si>
   <si>
     <t>Automation Stack</t>
@@ -2839,7 +2839,7 @@
         <v>47</v>
       </c>
       <c r="G2" s="13">
-        <v>2793</v>
+        <v>1677</v>
       </c>
       <c r="H2" s="17" t="s">
         <v>48</v>
@@ -2868,7 +2868,7 @@
         <v>47</v>
       </c>
       <c r="G3" s="18">
-        <v>6451</v>
+        <v>3632</v>
       </c>
       <c r="H3" s="21" t="s">
         <v>48</v>
@@ -2897,7 +2897,7 @@
         <v>47</v>
       </c>
       <c r="G4" s="13">
-        <v>3686</v>
+        <v>8309</v>
       </c>
       <c r="H4" s="17" t="s">
         <v>48</v>
@@ -2926,7 +2926,7 @@
         <v>47</v>
       </c>
       <c r="G5" s="18">
-        <v>3866</v>
+        <v>2438</v>
       </c>
       <c r="H5" s="21" t="s">
         <v>48</v>
@@ -2955,7 +2955,7 @@
         <v>47</v>
       </c>
       <c r="G6" s="13">
-        <v>4138</v>
+        <v>6740</v>
       </c>
       <c r="H6" s="17" t="s">
         <v>48</v>
@@ -2984,7 +2984,7 @@
         <v>47</v>
       </c>
       <c r="G7" s="18">
-        <v>4662</v>
+        <v>1940</v>
       </c>
       <c r="H7" s="21" t="s">
         <v>48</v>
@@ -3013,7 +3013,7 @@
         <v>47</v>
       </c>
       <c r="G8" s="13">
-        <v>9041</v>
+        <v>3993</v>
       </c>
       <c r="H8" s="17" t="s">
         <v>48</v>
@@ -3042,7 +3042,7 @@
         <v>47</v>
       </c>
       <c r="G9" s="18">
-        <v>2094</v>
+        <v>3371</v>
       </c>
       <c r="H9" s="21" t="s">
         <v>48</v>
@@ -3071,7 +3071,7 @@
         <v>47</v>
       </c>
       <c r="G10" s="13">
-        <v>2388</v>
+        <v>1289</v>
       </c>
       <c r="H10" s="17" t="s">
         <v>48</v>
@@ -3100,7 +3100,7 @@
         <v>47</v>
       </c>
       <c r="G11" s="18">
-        <v>7289</v>
+        <v>2079</v>
       </c>
       <c r="H11" s="21" t="s">
         <v>48</v>
@@ -3129,7 +3129,7 @@
         <v>47</v>
       </c>
       <c r="G12" s="13">
-        <v>8295</v>
+        <v>3871</v>
       </c>
       <c r="H12" s="17" t="s">
         <v>48</v>
@@ -3158,7 +3158,7 @@
         <v>47</v>
       </c>
       <c r="G13" s="18">
-        <v>5169</v>
+        <v>3079</v>
       </c>
       <c r="H13" s="21" t="s">
         <v>48</v>
@@ -3187,7 +3187,7 @@
         <v>47</v>
       </c>
       <c r="G14" s="13">
-        <v>2420</v>
+        <v>1452</v>
       </c>
       <c r="H14" s="17" t="s">
         <v>48</v>
@@ -3216,7 +3216,7 @@
         <v>47</v>
       </c>
       <c r="G15" s="18">
-        <v>7102</v>
+        <v>5326</v>
       </c>
       <c r="H15" s="21" t="s">
         <v>48</v>
@@ -3245,7 +3245,7 @@
         <v>47</v>
       </c>
       <c r="G16" s="13">
-        <v>7391</v>
+        <v>6281</v>
       </c>
       <c r="H16" s="17" t="s">
         <v>48</v>
@@ -3274,7 +3274,7 @@
         <v>47</v>
       </c>
       <c r="G17" s="18">
-        <v>6031</v>
+        <v>5386</v>
       </c>
       <c r="H17" s="21" t="s">
         <v>48</v>
@@ -3303,7 +3303,7 @@
         <v>47</v>
       </c>
       <c r="G18" s="13">
-        <v>1750</v>
+        <v>4800</v>
       </c>
       <c r="H18" s="17" t="s">
         <v>48</v>
@@ -3332,7 +3332,7 @@
         <v>47</v>
       </c>
       <c r="G19" s="18">
-        <v>8586</v>
+        <v>8663</v>
       </c>
       <c r="H19" s="21" t="s">
         <v>48</v>
@@ -3361,7 +3361,7 @@
         <v>47</v>
       </c>
       <c r="G20" s="13">
-        <v>8128</v>
+        <v>8618</v>
       </c>
       <c r="H20" s="17" t="s">
         <v>48</v>
@@ -3390,7 +3390,7 @@
         <v>47</v>
       </c>
       <c r="G21" s="18">
-        <v>4159</v>
+        <v>5843</v>
       </c>
       <c r="H21" s="21" t="s">
         <v>48</v>
@@ -3419,7 +3419,7 @@
         <v>47</v>
       </c>
       <c r="G22" s="13">
-        <v>1308</v>
+        <v>7056</v>
       </c>
       <c r="H22" s="17" t="s">
         <v>48</v>
@@ -3448,7 +3448,7 @@
         <v>47</v>
       </c>
       <c r="G23" s="18">
-        <v>7744</v>
+        <v>2952</v>
       </c>
       <c r="H23" s="21" t="s">
         <v>48</v>
@@ -3477,7 +3477,7 @@
         <v>47</v>
       </c>
       <c r="G24" s="13">
-        <v>7721</v>
+        <v>5223</v>
       </c>
       <c r="H24" s="17" t="s">
         <v>48</v>
@@ -3506,7 +3506,7 @@
         <v>47</v>
       </c>
       <c r="G25" s="18">
-        <v>8723</v>
+        <v>8917</v>
       </c>
       <c r="H25" s="21" t="s">
         <v>48</v>
@@ -3535,7 +3535,7 @@
         <v>47</v>
       </c>
       <c r="G26" s="13">
-        <v>4346</v>
+        <v>8756</v>
       </c>
       <c r="H26" s="17" t="s">
         <v>48</v>
@@ -3564,7 +3564,7 @@
         <v>47</v>
       </c>
       <c r="G27" s="18">
-        <v>2739</v>
+        <v>5304</v>
       </c>
       <c r="H27" s="21" t="s">
         <v>48</v>
@@ -3593,7 +3593,7 @@
         <v>47</v>
       </c>
       <c r="G28" s="13">
-        <v>5858</v>
+        <v>2092</v>
       </c>
       <c r="H28" s="17" t="s">
         <v>48</v>
@@ -3622,7 +3622,7 @@
         <v>47</v>
       </c>
       <c r="G29" s="18">
-        <v>7758</v>
+        <v>2607</v>
       </c>
       <c r="H29" s="21" t="s">
         <v>48</v>
@@ -3651,7 +3651,7 @@
         <v>47</v>
       </c>
       <c r="G30" s="13">
-        <v>6038</v>
+        <v>7494</v>
       </c>
       <c r="H30" s="17" t="s">
         <v>48</v>
@@ -3680,7 +3680,7 @@
         <v>47</v>
       </c>
       <c r="G31" s="18">
-        <v>2505</v>
+        <v>5015</v>
       </c>
       <c r="H31" s="21" t="s">
         <v>48</v>
@@ -3709,7 +3709,7 @@
         <v>47</v>
       </c>
       <c r="G32" s="13">
-        <v>3760</v>
+        <v>7604</v>
       </c>
       <c r="H32" s="17" t="s">
         <v>48</v>
@@ -3738,7 +3738,7 @@
         <v>47</v>
       </c>
       <c r="G33" s="18">
-        <v>8938</v>
+        <v>2623</v>
       </c>
       <c r="H33" s="21" t="s">
         <v>48</v>
@@ -3767,7 +3767,7 @@
         <v>47</v>
       </c>
       <c r="G34" s="13">
-        <v>1931</v>
+        <v>2966</v>
       </c>
       <c r="H34" s="17" t="s">
         <v>48</v>
@@ -3796,7 +3796,7 @@
         <v>47</v>
       </c>
       <c r="G35" s="18">
-        <v>6992</v>
+        <v>6227</v>
       </c>
       <c r="H35" s="21" t="s">
         <v>48</v>
@@ -3825,7 +3825,7 @@
         <v>47</v>
       </c>
       <c r="G36" s="13">
-        <v>2217</v>
+        <v>3777</v>
       </c>
       <c r="H36" s="17" t="s">
         <v>48</v>
@@ -3854,7 +3854,7 @@
         <v>47</v>
       </c>
       <c r="G37" s="18">
-        <v>8466</v>
+        <v>5417</v>
       </c>
       <c r="H37" s="21" t="s">
         <v>48</v>
@@ -3883,7 +3883,7 @@
         <v>47</v>
       </c>
       <c r="G38" s="13">
-        <v>6608</v>
+        <v>6228</v>
       </c>
       <c r="H38" s="17" t="s">
         <v>48</v>
@@ -3912,7 +3912,7 @@
         <v>47</v>
       </c>
       <c r="G39" s="18">
-        <v>7328</v>
+        <v>8984</v>
       </c>
       <c r="H39" s="21" t="s">
         <v>48</v>
@@ -3941,7 +3941,7 @@
         <v>47</v>
       </c>
       <c r="G40" s="13">
-        <v>3085</v>
+        <v>7284</v>
       </c>
       <c r="H40" s="17" t="s">
         <v>48</v>
@@ -3970,7 +3970,7 @@
         <v>47</v>
       </c>
       <c r="G41" s="18">
-        <v>1822</v>
+        <v>2727</v>
       </c>
       <c r="H41" s="21" t="s">
         <v>48</v>
@@ -3999,7 +3999,7 @@
         <v>131</v>
       </c>
       <c r="G42" s="13">
-        <v>2372</v>
+        <v>3521</v>
       </c>
       <c r="H42" s="17" t="s">
         <v>48</v>
@@ -4028,7 +4028,7 @@
         <v>131</v>
       </c>
       <c r="G43" s="18">
-        <v>4058</v>
+        <v>8147</v>
       </c>
       <c r="H43" s="21" t="s">
         <v>48</v>
@@ -4057,7 +4057,7 @@
         <v>131</v>
       </c>
       <c r="G44" s="13">
-        <v>8517</v>
+        <v>2336</v>
       </c>
       <c r="H44" s="17" t="s">
         <v>48</v>
@@ -4086,7 +4086,7 @@
         <v>131</v>
       </c>
       <c r="G45" s="18">
-        <v>4091</v>
+        <v>4220</v>
       </c>
       <c r="H45" s="21" t="s">
         <v>48</v>
@@ -4115,7 +4115,7 @@
         <v>131</v>
       </c>
       <c r="G46" s="13">
-        <v>5027</v>
+        <v>9188</v>
       </c>
       <c r="H46" s="17" t="s">
         <v>48</v>
@@ -4144,7 +4144,7 @@
         <v>131</v>
       </c>
       <c r="G47" s="18">
-        <v>6601</v>
+        <v>2280</v>
       </c>
       <c r="H47" s="21" t="s">
         <v>48</v>
@@ -4173,7 +4173,7 @@
         <v>131</v>
       </c>
       <c r="G48" s="13">
-        <v>2858</v>
+        <v>2737</v>
       </c>
       <c r="H48" s="17" t="s">
         <v>48</v>
@@ -4202,7 +4202,7 @@
         <v>131</v>
       </c>
       <c r="G49" s="18">
-        <v>5667</v>
+        <v>2753</v>
       </c>
       <c r="H49" s="21" t="s">
         <v>48</v>
@@ -4231,7 +4231,7 @@
         <v>131</v>
       </c>
       <c r="G50" s="13">
-        <v>4052</v>
+        <v>1435</v>
       </c>
       <c r="H50" s="17" t="s">
         <v>48</v>
@@ -4260,7 +4260,7 @@
         <v>131</v>
       </c>
       <c r="G51" s="18">
-        <v>4812</v>
+        <v>5186</v>
       </c>
       <c r="H51" s="21" t="s">
         <v>48</v>
@@ -4289,7 +4289,7 @@
         <v>131</v>
       </c>
       <c r="G52" s="13">
-        <v>7101</v>
+        <v>1709</v>
       </c>
       <c r="H52" s="17" t="s">
         <v>48</v>
@@ -4318,7 +4318,7 @@
         <v>131</v>
       </c>
       <c r="G53" s="18">
-        <v>6152</v>
+        <v>2256</v>
       </c>
       <c r="H53" s="21" t="s">
         <v>48</v>
@@ -4347,7 +4347,7 @@
         <v>131</v>
       </c>
       <c r="G54" s="13">
-        <v>6085</v>
+        <v>5425</v>
       </c>
       <c r="H54" s="17" t="s">
         <v>48</v>
@@ -4376,7 +4376,7 @@
         <v>131</v>
       </c>
       <c r="G55" s="18">
-        <v>8461</v>
+        <v>2457</v>
       </c>
       <c r="H55" s="21" t="s">
         <v>48</v>
@@ -4405,7 +4405,7 @@
         <v>131</v>
       </c>
       <c r="G56" s="13">
-        <v>4937</v>
+        <v>2456</v>
       </c>
       <c r="H56" s="17" t="s">
         <v>48</v>
@@ -4434,7 +4434,7 @@
         <v>131</v>
       </c>
       <c r="G57" s="18">
-        <v>6499</v>
+        <v>5615</v>
       </c>
       <c r="H57" s="21" t="s">
         <v>48</v>
@@ -4463,7 +4463,7 @@
         <v>131</v>
       </c>
       <c r="G58" s="13">
-        <v>2681</v>
+        <v>6751</v>
       </c>
       <c r="H58" s="17" t="s">
         <v>48</v>
@@ -4492,7 +4492,7 @@
         <v>131</v>
       </c>
       <c r="G59" s="18">
-        <v>7455</v>
+        <v>6516</v>
       </c>
       <c r="H59" s="21" t="s">
         <v>48</v>
@@ -4521,7 +4521,7 @@
         <v>131</v>
       </c>
       <c r="G60" s="13">
-        <v>3255</v>
+        <v>1826</v>
       </c>
       <c r="H60" s="17" t="s">
         <v>48</v>
@@ -4550,7 +4550,7 @@
         <v>131</v>
       </c>
       <c r="G61" s="18">
-        <v>7922</v>
+        <v>2712</v>
       </c>
       <c r="H61" s="21" t="s">
         <v>48</v>
@@ -4579,7 +4579,7 @@
         <v>131</v>
       </c>
       <c r="G62" s="13">
-        <v>6195</v>
+        <v>7823</v>
       </c>
       <c r="H62" s="17" t="s">
         <v>48</v>
@@ -4608,7 +4608,7 @@
         <v>131</v>
       </c>
       <c r="G63" s="18">
-        <v>8806</v>
+        <v>6230</v>
       </c>
       <c r="H63" s="21" t="s">
         <v>48</v>
@@ -4637,7 +4637,7 @@
         <v>131</v>
       </c>
       <c r="G64" s="13">
-        <v>6233</v>
+        <v>5019</v>
       </c>
       <c r="H64" s="17" t="s">
         <v>48</v>
@@ -4666,7 +4666,7 @@
         <v>131</v>
       </c>
       <c r="G65" s="18">
-        <v>1942</v>
+        <v>4588</v>
       </c>
       <c r="H65" s="21" t="s">
         <v>48</v>
@@ -4695,7 +4695,7 @@
         <v>131</v>
       </c>
       <c r="G66" s="13">
-        <v>3326</v>
+        <v>3012</v>
       </c>
       <c r="H66" s="17" t="s">
         <v>48</v>
@@ -4724,7 +4724,7 @@
         <v>131</v>
       </c>
       <c r="G67" s="18">
-        <v>4158</v>
+        <v>5630</v>
       </c>
       <c r="H67" s="21" t="s">
         <v>48</v>
@@ -4753,7 +4753,7 @@
         <v>131</v>
       </c>
       <c r="G68" s="13">
-        <v>2195</v>
+        <v>3290</v>
       </c>
       <c r="H68" s="17" t="s">
         <v>48</v>
@@ -4782,7 +4782,7 @@
         <v>131</v>
       </c>
       <c r="G69" s="18">
-        <v>3735</v>
+        <v>8937</v>
       </c>
       <c r="H69" s="21" t="s">
         <v>48</v>
@@ -4811,7 +4811,7 @@
         <v>131</v>
       </c>
       <c r="G70" s="13">
-        <v>1795</v>
+        <v>8901</v>
       </c>
       <c r="H70" s="17" t="s">
         <v>48</v>
@@ -4840,7 +4840,7 @@
         <v>131</v>
       </c>
       <c r="G71" s="18">
-        <v>3818</v>
+        <v>4988</v>
       </c>
       <c r="H71" s="21" t="s">
         <v>48</v>
@@ -4869,7 +4869,7 @@
         <v>131</v>
       </c>
       <c r="G72" s="13">
-        <v>1502</v>
+        <v>6085</v>
       </c>
       <c r="H72" s="17" t="s">
         <v>48</v>
@@ -4898,7 +4898,7 @@
         <v>131</v>
       </c>
       <c r="G73" s="18">
-        <v>3531</v>
+        <v>2225</v>
       </c>
       <c r="H73" s="21" t="s">
         <v>48</v>
@@ -4927,7 +4927,7 @@
         <v>131</v>
       </c>
       <c r="G74" s="13">
-        <v>2669</v>
+        <v>5211</v>
       </c>
       <c r="H74" s="17" t="s">
         <v>48</v>
@@ -4956,7 +4956,7 @@
         <v>131</v>
       </c>
       <c r="G75" s="18">
-        <v>2216</v>
+        <v>3968</v>
       </c>
       <c r="H75" s="21" t="s">
         <v>48</v>
@@ -4985,7 +4985,7 @@
         <v>131</v>
       </c>
       <c r="G76" s="13">
-        <v>5687</v>
+        <v>8398</v>
       </c>
       <c r="H76" s="17" t="s">
         <v>48</v>
@@ -5014,7 +5014,7 @@
         <v>131</v>
       </c>
       <c r="G77" s="18">
-        <v>3660</v>
+        <v>6340</v>
       </c>
       <c r="H77" s="21" t="s">
         <v>48</v>
@@ -5043,7 +5043,7 @@
         <v>131</v>
       </c>
       <c r="G78" s="13">
-        <v>2502</v>
+        <v>9086</v>
       </c>
       <c r="H78" s="17" t="s">
         <v>48</v>
@@ -5072,7 +5072,7 @@
         <v>131</v>
       </c>
       <c r="G79" s="18">
-        <v>5493</v>
+        <v>7574</v>
       </c>
       <c r="H79" s="21" t="s">
         <v>48</v>
@@ -5101,7 +5101,7 @@
         <v>131</v>
       </c>
       <c r="G80" s="13">
-        <v>6218</v>
+        <v>2650</v>
       </c>
       <c r="H80" s="17" t="s">
         <v>48</v>
@@ -5130,7 +5130,7 @@
         <v>131</v>
       </c>
       <c r="G81" s="18">
-        <v>7492</v>
+        <v>2798</v>
       </c>
       <c r="H81" s="21" t="s">
         <v>48</v>
@@ -5159,7 +5159,7 @@
         <v>47</v>
       </c>
       <c r="G82" s="13">
-        <v>3512</v>
+        <v>7544</v>
       </c>
       <c r="H82" s="17" t="s">
         <v>48</v>
@@ -5188,7 +5188,7 @@
         <v>47</v>
       </c>
       <c r="G83" s="18">
-        <v>7688</v>
+        <v>4838</v>
       </c>
       <c r="H83" s="21" t="s">
         <v>48</v>
@@ -5217,7 +5217,7 @@
         <v>47</v>
       </c>
       <c r="G84" s="13">
-        <v>7006</v>
+        <v>7502</v>
       </c>
       <c r="H84" s="17" t="s">
         <v>48</v>
@@ -5246,7 +5246,7 @@
         <v>47</v>
       </c>
       <c r="G85" s="18">
-        <v>6041</v>
+        <v>1307</v>
       </c>
       <c r="H85" s="21" t="s">
         <v>48</v>
@@ -5275,7 +5275,7 @@
         <v>47</v>
       </c>
       <c r="G86" s="13">
-        <v>3759</v>
+        <v>7835</v>
       </c>
       <c r="H86" s="17" t="s">
         <v>48</v>
@@ -5304,7 +5304,7 @@
         <v>47</v>
       </c>
       <c r="G87" s="18">
-        <v>4092</v>
+        <v>1987</v>
       </c>
       <c r="H87" s="21" t="s">
         <v>48</v>
@@ -5333,7 +5333,7 @@
         <v>47</v>
       </c>
       <c r="G88" s="13">
-        <v>5966</v>
+        <v>8663</v>
       </c>
       <c r="H88" s="17" t="s">
         <v>48</v>
@@ -5362,7 +5362,7 @@
         <v>47</v>
       </c>
       <c r="G89" s="18">
-        <v>7997</v>
+        <v>3025</v>
       </c>
       <c r="H89" s="21" t="s">
         <v>48</v>
@@ -5391,7 +5391,7 @@
         <v>47</v>
       </c>
       <c r="G90" s="13">
-        <v>4411</v>
+        <v>2570</v>
       </c>
       <c r="H90" s="17" t="s">
         <v>48</v>
@@ -5420,7 +5420,7 @@
         <v>47</v>
       </c>
       <c r="G91" s="18">
-        <v>8798</v>
+        <v>5952</v>
       </c>
       <c r="H91" s="21" t="s">
         <v>48</v>
@@ -5449,7 +5449,7 @@
         <v>47</v>
       </c>
       <c r="G92" s="13">
-        <v>4760</v>
+        <v>3130</v>
       </c>
       <c r="H92" s="17" t="s">
         <v>48</v>
@@ -5478,7 +5478,7 @@
         <v>47</v>
       </c>
       <c r="G93" s="18">
-        <v>8379</v>
+        <v>7705</v>
       </c>
       <c r="H93" s="21" t="s">
         <v>48</v>
@@ -5507,7 +5507,7 @@
         <v>47</v>
       </c>
       <c r="G94" s="13">
-        <v>3110</v>
+        <v>4382</v>
       </c>
       <c r="H94" s="17" t="s">
         <v>48</v>
@@ -5536,7 +5536,7 @@
         <v>47</v>
       </c>
       <c r="G95" s="18">
-        <v>8733</v>
+        <v>7555</v>
       </c>
       <c r="H95" s="21" t="s">
         <v>48</v>
@@ -5565,7 +5565,7 @@
         <v>47</v>
       </c>
       <c r="G96" s="13">
-        <v>6968</v>
+        <v>5923</v>
       </c>
       <c r="H96" s="17" t="s">
         <v>48</v>
@@ -5594,7 +5594,7 @@
         <v>47</v>
       </c>
       <c r="G97" s="18">
-        <v>4163</v>
+        <v>8011</v>
       </c>
       <c r="H97" s="21" t="s">
         <v>48</v>
@@ -5623,7 +5623,7 @@
         <v>47</v>
       </c>
       <c r="G98" s="13">
-        <v>8497</v>
+        <v>8438</v>
       </c>
       <c r="H98" s="17" t="s">
         <v>48</v>
@@ -5652,7 +5652,7 @@
         <v>47</v>
       </c>
       <c r="G99" s="18">
-        <v>6491</v>
+        <v>4656</v>
       </c>
       <c r="H99" s="21" t="s">
         <v>48</v>
@@ -5681,7 +5681,7 @@
         <v>47</v>
       </c>
       <c r="G100" s="13">
-        <v>1827</v>
+        <v>5644</v>
       </c>
       <c r="H100" s="17" t="s">
         <v>48</v>
@@ -5710,7 +5710,7 @@
         <v>47</v>
       </c>
       <c r="G101" s="18">
-        <v>5966</v>
+        <v>7814</v>
       </c>
       <c r="H101" s="21" t="s">
         <v>48</v>
@@ -5739,7 +5739,7 @@
         <v>47</v>
       </c>
       <c r="G102" s="13">
-        <v>2009</v>
+        <v>4439</v>
       </c>
       <c r="H102" s="17" t="s">
         <v>48</v>
@@ -5768,7 +5768,7 @@
         <v>47</v>
       </c>
       <c r="G103" s="18">
-        <v>7698</v>
+        <v>1697</v>
       </c>
       <c r="H103" s="21" t="s">
         <v>48</v>
@@ -5797,7 +5797,7 @@
         <v>47</v>
       </c>
       <c r="G104" s="13">
-        <v>5306</v>
+        <v>7902</v>
       </c>
       <c r="H104" s="17" t="s">
         <v>48</v>
@@ -5826,7 +5826,7 @@
         <v>47</v>
       </c>
       <c r="G105" s="18">
-        <v>6530</v>
+        <v>3670</v>
       </c>
       <c r="H105" s="21" t="s">
         <v>48</v>
@@ -5855,7 +5855,7 @@
         <v>47</v>
       </c>
       <c r="G106" s="13">
-        <v>3088</v>
+        <v>4796</v>
       </c>
       <c r="H106" s="17" t="s">
         <v>48</v>
@@ -5884,7 +5884,7 @@
         <v>47</v>
       </c>
       <c r="G107" s="18">
-        <v>6737</v>
+        <v>2353</v>
       </c>
       <c r="H107" s="21" t="s">
         <v>48</v>
@@ -5913,7 +5913,7 @@
         <v>47</v>
       </c>
       <c r="G108" s="13">
-        <v>1776</v>
+        <v>3848</v>
       </c>
       <c r="H108" s="17" t="s">
         <v>48</v>
@@ -5942,7 +5942,7 @@
         <v>47</v>
       </c>
       <c r="G109" s="18">
-        <v>3241</v>
+        <v>6007</v>
       </c>
       <c r="H109" s="21" t="s">
         <v>48</v>
@@ -5971,7 +5971,7 @@
         <v>47</v>
       </c>
       <c r="G110" s="13">
-        <v>4758</v>
+        <v>5550</v>
       </c>
       <c r="H110" s="17" t="s">
         <v>48</v>
@@ -6000,7 +6000,7 @@
         <v>47</v>
       </c>
       <c r="G111" s="18">
-        <v>2927</v>
+        <v>3140</v>
       </c>
       <c r="H111" s="21" t="s">
         <v>48</v>
@@ -6029,7 +6029,7 @@
         <v>47</v>
       </c>
       <c r="G112" s="13">
-        <v>8068</v>
+        <v>5804</v>
       </c>
       <c r="H112" s="17" t="s">
         <v>48</v>
@@ -6058,7 +6058,7 @@
         <v>47</v>
       </c>
       <c r="G113" s="18">
-        <v>5682</v>
+        <v>2217</v>
       </c>
       <c r="H113" s="21" t="s">
         <v>48</v>
@@ -6087,7 +6087,7 @@
         <v>47</v>
       </c>
       <c r="G114" s="13">
-        <v>6361</v>
+        <v>2362</v>
       </c>
       <c r="H114" s="17" t="s">
         <v>48</v>
@@ -6116,7 +6116,7 @@
         <v>47</v>
       </c>
       <c r="G115" s="18">
-        <v>4029</v>
+        <v>6502</v>
       </c>
       <c r="H115" s="21" t="s">
         <v>48</v>
@@ -6145,7 +6145,7 @@
         <v>47</v>
       </c>
       <c r="G116" s="13">
-        <v>3885</v>
+        <v>6102</v>
       </c>
       <c r="H116" s="17" t="s">
         <v>48</v>
@@ -6174,7 +6174,7 @@
         <v>47</v>
       </c>
       <c r="G117" s="18">
-        <v>5621</v>
+        <v>4027</v>
       </c>
       <c r="H117" s="21" t="s">
         <v>48</v>
@@ -6203,7 +6203,7 @@
         <v>47</v>
       </c>
       <c r="G118" s="13">
-        <v>4662</v>
+        <v>5239</v>
       </c>
       <c r="H118" s="17" t="s">
         <v>48</v>
@@ -6232,7 +6232,7 @@
         <v>47</v>
       </c>
       <c r="G119" s="18">
-        <v>5007</v>
+        <v>4133</v>
       </c>
       <c r="H119" s="21" t="s">
         <v>48</v>
@@ -6261,7 +6261,7 @@
         <v>47</v>
       </c>
       <c r="G120" s="13">
-        <v>3338</v>
+        <v>3116</v>
       </c>
       <c r="H120" s="17" t="s">
         <v>48</v>
@@ -6290,7 +6290,7 @@
         <v>47</v>
       </c>
       <c r="G121" s="18">
-        <v>9142</v>
+        <v>4265</v>
       </c>
       <c r="H121" s="21" t="s">
         <v>48</v>
@@ -6319,7 +6319,7 @@
         <v>47</v>
       </c>
       <c r="G122" s="13">
-        <v>4656</v>
+        <v>6918</v>
       </c>
       <c r="H122" s="17" t="s">
         <v>48</v>
@@ -6348,7 +6348,7 @@
         <v>47</v>
       </c>
       <c r="G123" s="18">
-        <v>3892</v>
+        <v>3084</v>
       </c>
       <c r="H123" s="21" t="s">
         <v>48</v>
@@ -6377,7 +6377,7 @@
         <v>47</v>
       </c>
       <c r="G124" s="13">
-        <v>4859</v>
+        <v>7067</v>
       </c>
       <c r="H124" s="17" t="s">
         <v>48</v>
@@ -6406,7 +6406,7 @@
         <v>47</v>
       </c>
       <c r="G125" s="18">
-        <v>8671</v>
+        <v>9159</v>
       </c>
       <c r="H125" s="21" t="s">
         <v>48</v>
@@ -6435,7 +6435,7 @@
         <v>47</v>
       </c>
       <c r="G126" s="13">
-        <v>4071</v>
+        <v>7744</v>
       </c>
       <c r="H126" s="17" t="s">
         <v>48</v>
@@ -6464,7 +6464,7 @@
         <v>47</v>
       </c>
       <c r="G127" s="18">
-        <v>7500</v>
+        <v>4965</v>
       </c>
       <c r="H127" s="21" t="s">
         <v>48</v>
@@ -6493,7 +6493,7 @@
         <v>47</v>
       </c>
       <c r="G128" s="13">
-        <v>2736</v>
+        <v>2853</v>
       </c>
       <c r="H128" s="17" t="s">
         <v>48</v>
@@ -6522,7 +6522,7 @@
         <v>47</v>
       </c>
       <c r="G129" s="18">
-        <v>7161</v>
+        <v>9075</v>
       </c>
       <c r="H129" s="21" t="s">
         <v>48</v>
@@ -6551,7 +6551,7 @@
         <v>47</v>
       </c>
       <c r="G130" s="13">
-        <v>3667</v>
+        <v>5637</v>
       </c>
       <c r="H130" s="17" t="s">
         <v>48</v>
@@ -6580,7 +6580,7 @@
         <v>47</v>
       </c>
       <c r="G131" s="18">
-        <v>7942</v>
+        <v>4973</v>
       </c>
       <c r="H131" s="21" t="s">
         <v>48</v>
@@ -6609,7 +6609,7 @@
         <v>47</v>
       </c>
       <c r="G132" s="13">
-        <v>3755</v>
+        <v>4244</v>
       </c>
       <c r="H132" s="17" t="s">
         <v>48</v>
@@ -6638,7 +6638,7 @@
         <v>47</v>
       </c>
       <c r="G133" s="18">
-        <v>5714</v>
+        <v>3750</v>
       </c>
       <c r="H133" s="21" t="s">
         <v>48</v>
@@ -6667,7 +6667,7 @@
         <v>47</v>
       </c>
       <c r="G134" s="13">
-        <v>8995</v>
+        <v>6491</v>
       </c>
       <c r="H134" s="17" t="s">
         <v>48</v>
@@ -6696,7 +6696,7 @@
         <v>47</v>
       </c>
       <c r="G135" s="18">
-        <v>1964</v>
+        <v>1912</v>
       </c>
       <c r="H135" s="21" t="s">
         <v>48</v>
@@ -6725,7 +6725,7 @@
         <v>47</v>
       </c>
       <c r="G136" s="13">
-        <v>8496</v>
+        <v>5514</v>
       </c>
       <c r="H136" s="17" t="s">
         <v>48</v>
@@ -6754,7 +6754,7 @@
         <v>47</v>
       </c>
       <c r="G137" s="18">
-        <v>6474</v>
+        <v>6758</v>
       </c>
       <c r="H137" s="21" t="s">
         <v>48</v>
@@ -6783,7 +6783,7 @@
         <v>47</v>
       </c>
       <c r="G138" s="13">
-        <v>5561</v>
+        <v>8720</v>
       </c>
       <c r="H138" s="17" t="s">
         <v>48</v>
@@ -6812,7 +6812,7 @@
         <v>47</v>
       </c>
       <c r="G139" s="18">
-        <v>4767</v>
+        <v>4719</v>
       </c>
       <c r="H139" s="21" t="s">
         <v>48</v>
@@ -6841,7 +6841,7 @@
         <v>47</v>
       </c>
       <c r="G140" s="13">
-        <v>6145</v>
+        <v>7957</v>
       </c>
       <c r="H140" s="17" t="s">
         <v>48</v>
@@ -6870,7 +6870,7 @@
         <v>47</v>
       </c>
       <c r="G141" s="18">
-        <v>8075</v>
+        <v>5602</v>
       </c>
       <c r="H141" s="21" t="s">
         <v>48</v>
@@ -6899,7 +6899,7 @@
         <v>47</v>
       </c>
       <c r="G142" s="13">
-        <v>2409</v>
+        <v>7690</v>
       </c>
       <c r="H142" s="17" t="s">
         <v>48</v>
@@ -6928,7 +6928,7 @@
         <v>47</v>
       </c>
       <c r="G143" s="18">
-        <v>2990</v>
+        <v>5005</v>
       </c>
       <c r="H143" s="21" t="s">
         <v>48</v>
@@ -6957,7 +6957,7 @@
         <v>47</v>
       </c>
       <c r="G144" s="13">
-        <v>6243</v>
+        <v>8871</v>
       </c>
       <c r="H144" s="17" t="s">
         <v>48</v>
@@ -6986,7 +6986,7 @@
         <v>47</v>
       </c>
       <c r="G145" s="18">
-        <v>2112</v>
+        <v>4006</v>
       </c>
       <c r="H145" s="21" t="s">
         <v>48</v>
@@ -7015,7 +7015,7 @@
         <v>47</v>
       </c>
       <c r="G146" s="13">
-        <v>3277</v>
+        <v>7738</v>
       </c>
       <c r="H146" s="17" t="s">
         <v>48</v>
@@ -7044,7 +7044,7 @@
         <v>47</v>
       </c>
       <c r="G147" s="18">
-        <v>5325</v>
+        <v>6719</v>
       </c>
       <c r="H147" s="21" t="s">
         <v>48</v>
@@ -7073,7 +7073,7 @@
         <v>47</v>
       </c>
       <c r="G148" s="13">
-        <v>6704</v>
+        <v>1283</v>
       </c>
       <c r="H148" s="17" t="s">
         <v>48</v>
@@ -7102,7 +7102,7 @@
         <v>47</v>
       </c>
       <c r="G149" s="18">
-        <v>5943</v>
+        <v>7921</v>
       </c>
       <c r="H149" s="21" t="s">
         <v>48</v>
@@ -7131,7 +7131,7 @@
         <v>47</v>
       </c>
       <c r="G150" s="13">
-        <v>3797</v>
+        <v>6349</v>
       </c>
       <c r="H150" s="17" t="s">
         <v>48</v>
@@ -7160,7 +7160,7 @@
         <v>47</v>
       </c>
       <c r="G151" s="18">
-        <v>2223</v>
+        <v>4961</v>
       </c>
       <c r="H151" s="21" t="s">
         <v>48</v>
@@ -7189,7 +7189,7 @@
         <v>47</v>
       </c>
       <c r="G152" s="13">
-        <v>8781</v>
+        <v>6656</v>
       </c>
       <c r="H152" s="17" t="s">
         <v>48</v>
@@ -7218,7 +7218,7 @@
         <v>47</v>
       </c>
       <c r="G153" s="18">
-        <v>8907</v>
+        <v>2685</v>
       </c>
       <c r="H153" s="21" t="s">
         <v>48</v>
@@ -7247,7 +7247,7 @@
         <v>47</v>
       </c>
       <c r="G154" s="13">
-        <v>8544</v>
+        <v>8562</v>
       </c>
       <c r="H154" s="17" t="s">
         <v>48</v>
@@ -7276,7 +7276,7 @@
         <v>47</v>
       </c>
       <c r="G155" s="18">
-        <v>2673</v>
+        <v>5060</v>
       </c>
       <c r="H155" s="21" t="s">
         <v>48</v>
@@ -7305,7 +7305,7 @@
         <v>47</v>
       </c>
       <c r="G156" s="13">
-        <v>2115</v>
+        <v>6875</v>
       </c>
       <c r="H156" s="17" t="s">
         <v>48</v>
@@ -7334,7 +7334,7 @@
         <v>47</v>
       </c>
       <c r="G157" s="18">
-        <v>7410</v>
+        <v>2453</v>
       </c>
       <c r="H157" s="21" t="s">
         <v>48</v>
@@ -7363,7 +7363,7 @@
         <v>47</v>
       </c>
       <c r="G158" s="13">
-        <v>1469</v>
+        <v>1683</v>
       </c>
       <c r="H158" s="17" t="s">
         <v>48</v>
@@ -7392,7 +7392,7 @@
         <v>47</v>
       </c>
       <c r="G159" s="18">
-        <v>6004</v>
+        <v>1994</v>
       </c>
       <c r="H159" s="21" t="s">
         <v>48</v>
@@ -7421,7 +7421,7 @@
         <v>47</v>
       </c>
       <c r="G160" s="13">
-        <v>5367</v>
+        <v>1727</v>
       </c>
       <c r="H160" s="17" t="s">
         <v>48</v>
@@ -7450,7 +7450,7 @@
         <v>47</v>
       </c>
       <c r="G161" s="18">
-        <v>4775</v>
+        <v>5009</v>
       </c>
       <c r="H161" s="21" t="s">
         <v>48</v>
@@ -7479,7 +7479,7 @@
         <v>47</v>
       </c>
       <c r="G162" s="13">
-        <v>3291</v>
+        <v>7087</v>
       </c>
       <c r="H162" s="17" t="s">
         <v>48</v>
@@ -7508,7 +7508,7 @@
         <v>47</v>
       </c>
       <c r="G163" s="18">
-        <v>1751</v>
+        <v>4260</v>
       </c>
       <c r="H163" s="21" t="s">
         <v>48</v>
@@ -7537,7 +7537,7 @@
         <v>47</v>
       </c>
       <c r="G164" s="13">
-        <v>4161</v>
+        <v>3458</v>
       </c>
       <c r="H164" s="17" t="s">
         <v>48</v>
@@ -7566,7 +7566,7 @@
         <v>47</v>
       </c>
       <c r="G165" s="18">
-        <v>5389</v>
+        <v>3387</v>
       </c>
       <c r="H165" s="21" t="s">
         <v>48</v>
@@ -7595,7 +7595,7 @@
         <v>47</v>
       </c>
       <c r="G166" s="13">
-        <v>6231</v>
+        <v>7573</v>
       </c>
       <c r="H166" s="17" t="s">
         <v>48</v>
@@ -7624,7 +7624,7 @@
         <v>47</v>
       </c>
       <c r="G167" s="18">
-        <v>5177</v>
+        <v>3677</v>
       </c>
       <c r="H167" s="21" t="s">
         <v>48</v>
@@ -7653,7 +7653,7 @@
         <v>47</v>
       </c>
       <c r="G168" s="13">
-        <v>1268</v>
+        <v>3608</v>
       </c>
       <c r="H168" s="17" t="s">
         <v>48</v>
@@ -7682,7 +7682,7 @@
         <v>47</v>
       </c>
       <c r="G169" s="18">
-        <v>8989</v>
+        <v>2313</v>
       </c>
       <c r="H169" s="21" t="s">
         <v>48</v>
@@ -7711,7 +7711,7 @@
         <v>47</v>
       </c>
       <c r="G170" s="13">
-        <v>2667</v>
+        <v>1926</v>
       </c>
       <c r="H170" s="17" t="s">
         <v>48</v>
@@ -7740,7 +7740,7 @@
         <v>47</v>
       </c>
       <c r="G171" s="18">
-        <v>7944</v>
+        <v>8370</v>
       </c>
       <c r="H171" s="21" t="s">
         <v>48</v>
@@ -7769,7 +7769,7 @@
         <v>47</v>
       </c>
       <c r="G172" s="13">
-        <v>2962</v>
+        <v>6808</v>
       </c>
       <c r="H172" s="17" t="s">
         <v>48</v>
@@ -7798,7 +7798,7 @@
         <v>47</v>
       </c>
       <c r="G173" s="18">
-        <v>5275</v>
+        <v>1572</v>
       </c>
       <c r="H173" s="21" t="s">
         <v>48</v>
@@ -7827,7 +7827,7 @@
         <v>47</v>
       </c>
       <c r="G174" s="13">
-        <v>6708</v>
+        <v>5643</v>
       </c>
       <c r="H174" s="17" t="s">
         <v>48</v>
@@ -7856,7 +7856,7 @@
         <v>47</v>
       </c>
       <c r="G175" s="18">
-        <v>4146</v>
+        <v>5985</v>
       </c>
       <c r="H175" s="21" t="s">
         <v>48</v>
@@ -7885,7 +7885,7 @@
         <v>47</v>
       </c>
       <c r="G176" s="13">
-        <v>8386</v>
+        <v>6390</v>
       </c>
       <c r="H176" s="17" t="s">
         <v>48</v>
@@ -7914,7 +7914,7 @@
         <v>47</v>
       </c>
       <c r="G177" s="18">
-        <v>6505</v>
+        <v>3030</v>
       </c>
       <c r="H177" s="21" t="s">
         <v>48</v>
@@ -7943,7 +7943,7 @@
         <v>47</v>
       </c>
       <c r="G178" s="13">
-        <v>3851</v>
+        <v>6140</v>
       </c>
       <c r="H178" s="17" t="s">
         <v>48</v>
@@ -7972,7 +7972,7 @@
         <v>47</v>
       </c>
       <c r="G179" s="18">
-        <v>2590</v>
+        <v>4887</v>
       </c>
       <c r="H179" s="21" t="s">
         <v>48</v>
@@ -8001,7 +8001,7 @@
         <v>47</v>
       </c>
       <c r="G180" s="13">
-        <v>4585</v>
+        <v>5123</v>
       </c>
       <c r="H180" s="17" t="s">
         <v>48</v>
@@ -8030,7 +8030,7 @@
         <v>47</v>
       </c>
       <c r="G181" s="18">
-        <v>2821</v>
+        <v>6798</v>
       </c>
       <c r="H181" s="21" t="s">
         <v>48</v>
@@ -8059,7 +8059,7 @@
         <v>47</v>
       </c>
       <c r="G182" s="13">
-        <v>3447</v>
+        <v>6024</v>
       </c>
       <c r="H182" s="17" t="s">
         <v>48</v>
@@ -8088,7 +8088,7 @@
         <v>47</v>
       </c>
       <c r="G183" s="18">
-        <v>5388</v>
+        <v>5089</v>
       </c>
       <c r="H183" s="21" t="s">
         <v>48</v>
@@ -8117,7 +8117,7 @@
         <v>47</v>
       </c>
       <c r="G184" s="13">
-        <v>5240</v>
+        <v>4778</v>
       </c>
       <c r="H184" s="17" t="s">
         <v>48</v>
@@ -8146,7 +8146,7 @@
         <v>47</v>
       </c>
       <c r="G185" s="18">
-        <v>2265</v>
+        <v>8289</v>
       </c>
       <c r="H185" s="21" t="s">
         <v>48</v>
@@ -8175,7 +8175,7 @@
         <v>47</v>
       </c>
       <c r="G186" s="13">
-        <v>8289</v>
+        <v>3182</v>
       </c>
       <c r="H186" s="17" t="s">
         <v>48</v>
@@ -8204,7 +8204,7 @@
         <v>47</v>
       </c>
       <c r="G187" s="18">
-        <v>4448</v>
+        <v>2117</v>
       </c>
       <c r="H187" s="21" t="s">
         <v>48</v>
@@ -8233,7 +8233,7 @@
         <v>47</v>
       </c>
       <c r="G188" s="13">
-        <v>6750</v>
+        <v>3544</v>
       </c>
       <c r="H188" s="17" t="s">
         <v>48</v>
@@ -8262,7 +8262,7 @@
         <v>47</v>
       </c>
       <c r="G189" s="18">
-        <v>5702</v>
+        <v>2516</v>
       </c>
       <c r="H189" s="21" t="s">
         <v>48</v>
@@ -8291,7 +8291,7 @@
         <v>47</v>
       </c>
       <c r="G190" s="13">
-        <v>8184</v>
+        <v>5791</v>
       </c>
       <c r="H190" s="17" t="s">
         <v>48</v>
@@ -8320,7 +8320,7 @@
         <v>47</v>
       </c>
       <c r="G191" s="18">
-        <v>1950</v>
+        <v>5107</v>
       </c>
       <c r="H191" s="21" t="s">
         <v>48</v>
@@ -8349,7 +8349,7 @@
         <v>436</v>
       </c>
       <c r="G192" s="13">
-        <v>1509</v>
+        <v>7774</v>
       </c>
       <c r="H192" s="17" t="s">
         <v>48</v>
@@ -8378,7 +8378,7 @@
         <v>436</v>
       </c>
       <c r="G193" s="18">
-        <v>8259</v>
+        <v>2839</v>
       </c>
       <c r="H193" s="21" t="s">
         <v>48</v>
@@ -8407,7 +8407,7 @@
         <v>436</v>
       </c>
       <c r="G194" s="13">
-        <v>2369</v>
+        <v>4826</v>
       </c>
       <c r="H194" s="17" t="s">
         <v>48</v>
@@ -8436,7 +8436,7 @@
         <v>436</v>
       </c>
       <c r="G195" s="18">
-        <v>3737</v>
+        <v>4199</v>
       </c>
       <c r="H195" s="21" t="s">
         <v>48</v>
@@ -8465,7 +8465,7 @@
         <v>436</v>
       </c>
       <c r="G196" s="13">
-        <v>2979</v>
+        <v>1789</v>
       </c>
       <c r="H196" s="17" t="s">
         <v>48</v>
@@ -8494,7 +8494,7 @@
         <v>436</v>
       </c>
       <c r="G197" s="18">
-        <v>6352</v>
+        <v>2113</v>
       </c>
       <c r="H197" s="21" t="s">
         <v>48</v>
@@ -8523,7 +8523,7 @@
         <v>436</v>
       </c>
       <c r="G198" s="13">
-        <v>1451</v>
+        <v>5826</v>
       </c>
       <c r="H198" s="17" t="s">
         <v>48</v>
@@ -8552,7 +8552,7 @@
         <v>436</v>
       </c>
       <c r="G199" s="18">
-        <v>8059</v>
+        <v>2545</v>
       </c>
       <c r="H199" s="21" t="s">
         <v>48</v>
@@ -8581,7 +8581,7 @@
         <v>436</v>
       </c>
       <c r="G200" s="13">
-        <v>2643</v>
+        <v>4125</v>
       </c>
       <c r="H200" s="17" t="s">
         <v>48</v>
@@ -8610,7 +8610,7 @@
         <v>436</v>
       </c>
       <c r="G201" s="18">
-        <v>2033</v>
+        <v>7988</v>
       </c>
       <c r="H201" s="21" t="s">
         <v>48</v>
@@ -8639,7 +8639,7 @@
         <v>436</v>
       </c>
       <c r="G202" s="13">
-        <v>1598</v>
+        <v>2236</v>
       </c>
       <c r="H202" s="17" t="s">
         <v>48</v>
@@ -8668,7 +8668,7 @@
         <v>436</v>
       </c>
       <c r="G203" s="18">
-        <v>7461</v>
+        <v>4529</v>
       </c>
       <c r="H203" s="21" t="s">
         <v>48</v>
@@ -8697,7 +8697,7 @@
         <v>436</v>
       </c>
       <c r="G204" s="13">
-        <v>7640</v>
+        <v>4862</v>
       </c>
       <c r="H204" s="17" t="s">
         <v>48</v>
@@ -8726,7 +8726,7 @@
         <v>436</v>
       </c>
       <c r="G205" s="18">
-        <v>6687</v>
+        <v>7524</v>
       </c>
       <c r="H205" s="21" t="s">
         <v>48</v>
@@ -8755,7 +8755,7 @@
         <v>436</v>
       </c>
       <c r="G206" s="13">
-        <v>1644</v>
+        <v>4702</v>
       </c>
       <c r="H206" s="17" t="s">
         <v>48</v>
@@ -8784,7 +8784,7 @@
         <v>436</v>
       </c>
       <c r="G207" s="18">
-        <v>1272</v>
+        <v>4740</v>
       </c>
       <c r="H207" s="21" t="s">
         <v>48</v>
@@ -8813,7 +8813,7 @@
         <v>436</v>
       </c>
       <c r="G208" s="13">
-        <v>5269</v>
+        <v>3577</v>
       </c>
       <c r="H208" s="17" t="s">
         <v>48</v>
@@ -8842,7 +8842,7 @@
         <v>436</v>
       </c>
       <c r="G209" s="18">
-        <v>1569</v>
+        <v>2415</v>
       </c>
       <c r="H209" s="21" t="s">
         <v>48</v>
@@ -8871,7 +8871,7 @@
         <v>436</v>
       </c>
       <c r="G210" s="13">
-        <v>9062</v>
+        <v>8583</v>
       </c>
       <c r="H210" s="17" t="s">
         <v>48</v>
@@ -8900,7 +8900,7 @@
         <v>436</v>
       </c>
       <c r="G211" s="18">
-        <v>7857</v>
+        <v>2148</v>
       </c>
       <c r="H211" s="21" t="s">
         <v>48</v>
@@ -8929,7 +8929,7 @@
         <v>436</v>
       </c>
       <c r="G212" s="13">
-        <v>8646</v>
+        <v>5530</v>
       </c>
       <c r="H212" s="17" t="s">
         <v>48</v>
@@ -8958,7 +8958,7 @@
         <v>436</v>
       </c>
       <c r="G213" s="18">
-        <v>2547</v>
+        <v>5162</v>
       </c>
       <c r="H213" s="21" t="s">
         <v>48</v>
@@ -8987,7 +8987,7 @@
         <v>436</v>
       </c>
       <c r="G214" s="13">
-        <v>2063</v>
+        <v>3658</v>
       </c>
       <c r="H214" s="17" t="s">
         <v>48</v>
@@ -9016,7 +9016,7 @@
         <v>436</v>
       </c>
       <c r="G215" s="18">
-        <v>2985</v>
+        <v>2963</v>
       </c>
       <c r="H215" s="21" t="s">
         <v>48</v>
@@ -9045,7 +9045,7 @@
         <v>436</v>
       </c>
       <c r="G216" s="13">
-        <v>9126</v>
+        <v>5173</v>
       </c>
       <c r="H216" s="17" t="s">
         <v>48</v>
@@ -9074,7 +9074,7 @@
         <v>436</v>
       </c>
       <c r="G217" s="18">
-        <v>2935</v>
+        <v>7995</v>
       </c>
       <c r="H217" s="21" t="s">
         <v>48</v>
@@ -9103,7 +9103,7 @@
         <v>436</v>
       </c>
       <c r="G218" s="13">
-        <v>1429</v>
+        <v>4267</v>
       </c>
       <c r="H218" s="17" t="s">
         <v>48</v>
@@ -9132,7 +9132,7 @@
         <v>436</v>
       </c>
       <c r="G219" s="18">
-        <v>8897</v>
+        <v>2485</v>
       </c>
       <c r="H219" s="21" t="s">
         <v>48</v>
@@ -9161,7 +9161,7 @@
         <v>436</v>
       </c>
       <c r="G220" s="13">
-        <v>2989</v>
+        <v>4267</v>
       </c>
       <c r="H220" s="17" t="s">
         <v>48</v>
@@ -9190,7 +9190,7 @@
         <v>436</v>
       </c>
       <c r="G221" s="18">
-        <v>1405</v>
+        <v>6403</v>
       </c>
       <c r="H221" s="21" t="s">
         <v>48</v>
@@ -9219,7 +9219,7 @@
         <v>436</v>
       </c>
       <c r="G222" s="13">
-        <v>2091</v>
+        <v>7641</v>
       </c>
       <c r="H222" s="17" t="s">
         <v>48</v>
@@ -9248,7 +9248,7 @@
         <v>436</v>
       </c>
       <c r="G223" s="18">
-        <v>5735</v>
+        <v>4894</v>
       </c>
       <c r="H223" s="21" t="s">
         <v>48</v>
@@ -9277,7 +9277,7 @@
         <v>436</v>
       </c>
       <c r="G224" s="13">
-        <v>4839</v>
+        <v>4028</v>
       </c>
       <c r="H224" s="17" t="s">
         <v>48</v>
@@ -9306,7 +9306,7 @@
         <v>436</v>
       </c>
       <c r="G225" s="18">
-        <v>7685</v>
+        <v>1678</v>
       </c>
       <c r="H225" s="21" t="s">
         <v>48</v>
@@ -9335,7 +9335,7 @@
         <v>436</v>
       </c>
       <c r="G226" s="13">
-        <v>2605</v>
+        <v>4259</v>
       </c>
       <c r="H226" s="17" t="s">
         <v>48</v>
@@ -9364,7 +9364,7 @@
         <v>436</v>
       </c>
       <c r="G227" s="18">
-        <v>8618</v>
+        <v>1473</v>
       </c>
       <c r="H227" s="21" t="s">
         <v>48</v>
@@ -9393,7 +9393,7 @@
         <v>436</v>
       </c>
       <c r="G228" s="13">
-        <v>4011</v>
+        <v>3136</v>
       </c>
       <c r="H228" s="17" t="s">
         <v>48</v>
@@ -9422,7 +9422,7 @@
         <v>436</v>
       </c>
       <c r="G229" s="18">
-        <v>2060</v>
+        <v>7085</v>
       </c>
       <c r="H229" s="21" t="s">
         <v>48</v>
@@ -9451,7 +9451,7 @@
         <v>436</v>
       </c>
       <c r="G230" s="13">
-        <v>5025</v>
+        <v>8553</v>
       </c>
       <c r="H230" s="17" t="s">
         <v>48</v>
@@ -9480,7 +9480,7 @@
         <v>436</v>
       </c>
       <c r="G231" s="18">
-        <v>3161</v>
+        <v>8502</v>
       </c>
       <c r="H231" s="21" t="s">
         <v>48</v>
@@ -9509,7 +9509,7 @@
         <v>47</v>
       </c>
       <c r="G232" s="13">
-        <v>6351</v>
+        <v>9125</v>
       </c>
       <c r="H232" s="17" t="s">
         <v>48</v>
@@ -9538,7 +9538,7 @@
         <v>47</v>
       </c>
       <c r="G233" s="18">
-        <v>2064</v>
+        <v>4542</v>
       </c>
       <c r="H233" s="21" t="s">
         <v>48</v>
@@ -9567,7 +9567,7 @@
         <v>47</v>
       </c>
       <c r="G234" s="13">
-        <v>3741</v>
+        <v>2086</v>
       </c>
       <c r="H234" s="17" t="s">
         <v>48</v>
@@ -9596,7 +9596,7 @@
         <v>47</v>
       </c>
       <c r="G235" s="18">
-        <v>2891</v>
+        <v>5834</v>
       </c>
       <c r="H235" s="21" t="s">
         <v>48</v>
@@ -9625,7 +9625,7 @@
         <v>47</v>
       </c>
       <c r="G236" s="13">
-        <v>8149</v>
+        <v>5731</v>
       </c>
       <c r="H236" s="17" t="s">
         <v>48</v>
@@ -9654,7 +9654,7 @@
         <v>47</v>
       </c>
       <c r="G237" s="18">
-        <v>1803</v>
+        <v>8735</v>
       </c>
       <c r="H237" s="21" t="s">
         <v>48</v>
@@ -9683,7 +9683,7 @@
         <v>47</v>
       </c>
       <c r="G238" s="13">
-        <v>2728</v>
+        <v>7313</v>
       </c>
       <c r="H238" s="17" t="s">
         <v>48</v>
@@ -9712,7 +9712,7 @@
         <v>47</v>
       </c>
       <c r="G239" s="18">
-        <v>5404</v>
+        <v>4857</v>
       </c>
       <c r="H239" s="21" t="s">
         <v>48</v>
@@ -9741,7 +9741,7 @@
         <v>47</v>
       </c>
       <c r="G240" s="13">
-        <v>7596</v>
+        <v>6187</v>
       </c>
       <c r="H240" s="17" t="s">
         <v>48</v>
@@ -9770,7 +9770,7 @@
         <v>47</v>
       </c>
       <c r="G241" s="18">
-        <v>2443</v>
+        <v>4640</v>
       </c>
       <c r="H241" s="21" t="s">
         <v>48</v>
@@ -9799,7 +9799,7 @@
         <v>47</v>
       </c>
       <c r="G242" s="13">
-        <v>4016</v>
+        <v>6612</v>
       </c>
       <c r="H242" s="17" t="s">
         <v>48</v>
@@ -9828,7 +9828,7 @@
         <v>47</v>
       </c>
       <c r="G243" s="18">
-        <v>7745</v>
+        <v>5325</v>
       </c>
       <c r="H243" s="21" t="s">
         <v>48</v>
@@ -9857,7 +9857,7 @@
         <v>47</v>
       </c>
       <c r="G244" s="13">
-        <v>5713</v>
+        <v>3063</v>
       </c>
       <c r="H244" s="17" t="s">
         <v>48</v>
@@ -9886,7 +9886,7 @@
         <v>47</v>
       </c>
       <c r="G245" s="18">
-        <v>2837</v>
+        <v>5903</v>
       </c>
       <c r="H245" s="21" t="s">
         <v>48</v>
@@ -9915,7 +9915,7 @@
         <v>47</v>
       </c>
       <c r="G246" s="13">
-        <v>7899</v>
+        <v>2057</v>
       </c>
       <c r="H246" s="17" t="s">
         <v>48</v>
@@ -9944,7 +9944,7 @@
         <v>47</v>
       </c>
       <c r="G247" s="18">
-        <v>4972</v>
+        <v>2245</v>
       </c>
       <c r="H247" s="21" t="s">
         <v>48</v>
@@ -9973,7 +9973,7 @@
         <v>47</v>
       </c>
       <c r="G248" s="13">
-        <v>3972</v>
+        <v>8644</v>
       </c>
       <c r="H248" s="17" t="s">
         <v>48</v>
@@ -10002,7 +10002,7 @@
         <v>47</v>
       </c>
       <c r="G249" s="18">
-        <v>3198</v>
+        <v>2591</v>
       </c>
       <c r="H249" s="21" t="s">
         <v>48</v>
@@ -10031,7 +10031,7 @@
         <v>47</v>
       </c>
       <c r="G250" s="13">
-        <v>8865</v>
+        <v>7022</v>
       </c>
       <c r="H250" s="17" t="s">
         <v>48</v>
@@ -10060,7 +10060,7 @@
         <v>47</v>
       </c>
       <c r="G251" s="18">
-        <v>4216</v>
+        <v>1234</v>
       </c>
       <c r="H251" s="21" t="s">
         <v>48</v>
@@ -10089,7 +10089,7 @@
         <v>47</v>
       </c>
       <c r="G252" s="13">
-        <v>1552</v>
+        <v>2330</v>
       </c>
       <c r="H252" s="17" t="s">
         <v>48</v>
@@ -10118,7 +10118,7 @@
         <v>47</v>
       </c>
       <c r="G253" s="18">
-        <v>2838</v>
+        <v>2608</v>
       </c>
       <c r="H253" s="21" t="s">
         <v>48</v>
@@ -10147,7 +10147,7 @@
         <v>47</v>
       </c>
       <c r="G254" s="13">
-        <v>3402</v>
+        <v>4718</v>
       </c>
       <c r="H254" s="17" t="s">
         <v>48</v>
@@ -10176,7 +10176,7 @@
         <v>47</v>
       </c>
       <c r="G255" s="18">
-        <v>5067</v>
+        <v>7803</v>
       </c>
       <c r="H255" s="21" t="s">
         <v>48</v>
@@ -10205,7 +10205,7 @@
         <v>47</v>
       </c>
       <c r="G256" s="13">
-        <v>8486</v>
+        <v>7607</v>
       </c>
       <c r="H256" s="17" t="s">
         <v>48</v>
@@ -10234,7 +10234,7 @@
         <v>47</v>
       </c>
       <c r="G257" s="18">
-        <v>5664</v>
+        <v>4666</v>
       </c>
       <c r="H257" s="21" t="s">
         <v>48</v>
@@ -10263,7 +10263,7 @@
         <v>47</v>
       </c>
       <c r="G258" s="13">
-        <v>3662</v>
+        <v>2688</v>
       </c>
       <c r="H258" s="17" t="s">
         <v>48</v>
@@ -10292,7 +10292,7 @@
         <v>47</v>
       </c>
       <c r="G259" s="18">
-        <v>8152</v>
+        <v>2042</v>
       </c>
       <c r="H259" s="21" t="s">
         <v>48</v>
@@ -10321,7 +10321,7 @@
         <v>47</v>
       </c>
       <c r="G260" s="13">
-        <v>1941</v>
+        <v>2384</v>
       </c>
       <c r="H260" s="17" t="s">
         <v>48</v>
@@ -10350,7 +10350,7 @@
         <v>47</v>
       </c>
       <c r="G261" s="18">
-        <v>6830</v>
+        <v>2568</v>
       </c>
       <c r="H261" s="21" t="s">
         <v>48</v>
@@ -10379,7 +10379,7 @@
         <v>47</v>
       </c>
       <c r="G262" s="13">
-        <v>3064</v>
+        <v>7177</v>
       </c>
       <c r="H262" s="17" t="s">
         <v>48</v>
@@ -10408,7 +10408,7 @@
         <v>47</v>
       </c>
       <c r="G263" s="18">
-        <v>3972</v>
+        <v>3181</v>
       </c>
       <c r="H263" s="21" t="s">
         <v>48</v>
@@ -10437,7 +10437,7 @@
         <v>47</v>
       </c>
       <c r="G264" s="13">
-        <v>4085</v>
+        <v>5937</v>
       </c>
       <c r="H264" s="17" t="s">
         <v>48</v>
@@ -10466,7 +10466,7 @@
         <v>47</v>
       </c>
       <c r="G265" s="18">
-        <v>1219</v>
+        <v>7382</v>
       </c>
       <c r="H265" s="21" t="s">
         <v>48</v>
@@ -10495,7 +10495,7 @@
         <v>47</v>
       </c>
       <c r="G266" s="13">
-        <v>3548</v>
+        <v>4142</v>
       </c>
       <c r="H266" s="17" t="s">
         <v>48</v>
@@ -10524,7 +10524,7 @@
         <v>47</v>
       </c>
       <c r="G267" s="18">
-        <v>5346</v>
+        <v>6227</v>
       </c>
       <c r="H267" s="21" t="s">
         <v>48</v>
@@ -10553,7 +10553,7 @@
         <v>47</v>
       </c>
       <c r="G268" s="13">
-        <v>8022</v>
+        <v>2726</v>
       </c>
       <c r="H268" s="17" t="s">
         <v>48</v>
@@ -10582,7 +10582,7 @@
         <v>47</v>
       </c>
       <c r="G269" s="18">
-        <v>7256</v>
+        <v>7692</v>
       </c>
       <c r="H269" s="21" t="s">
         <v>48</v>
@@ -10611,7 +10611,7 @@
         <v>47</v>
       </c>
       <c r="G270" s="13">
-        <v>2886</v>
+        <v>6105</v>
       </c>
       <c r="H270" s="17" t="s">
         <v>48</v>
@@ -10640,7 +10640,7 @@
         <v>47</v>
       </c>
       <c r="G271" s="18">
-        <v>4375</v>
+        <v>3584</v>
       </c>
       <c r="H271" s="21" t="s">
         <v>48</v>
@@ -10669,7 +10669,7 @@
         <v>47</v>
       </c>
       <c r="G272" s="13">
-        <v>3937</v>
+        <v>6855</v>
       </c>
       <c r="H272" s="17" t="s">
         <v>48</v>
@@ -10698,7 +10698,7 @@
         <v>47</v>
       </c>
       <c r="G273" s="18">
-        <v>6780</v>
+        <v>2944</v>
       </c>
       <c r="H273" s="21" t="s">
         <v>48</v>
@@ -10727,7 +10727,7 @@
         <v>47</v>
       </c>
       <c r="G274" s="13">
-        <v>6620</v>
+        <v>2501</v>
       </c>
       <c r="H274" s="17" t="s">
         <v>48</v>
@@ -10756,7 +10756,7 @@
         <v>47</v>
       </c>
       <c r="G275" s="18">
-        <v>1315</v>
+        <v>3566</v>
       </c>
       <c r="H275" s="21" t="s">
         <v>48</v>
@@ -10785,7 +10785,7 @@
         <v>47</v>
       </c>
       <c r="G276" s="13">
-        <v>4576</v>
+        <v>8176</v>
       </c>
       <c r="H276" s="17" t="s">
         <v>48</v>
@@ -10814,7 +10814,7 @@
         <v>47</v>
       </c>
       <c r="G277" s="18">
-        <v>6614</v>
+        <v>3897</v>
       </c>
       <c r="H277" s="21" t="s">
         <v>48</v>
@@ -10843,7 +10843,7 @@
         <v>47</v>
       </c>
       <c r="G278" s="13">
-        <v>6382</v>
+        <v>4426</v>
       </c>
       <c r="H278" s="17" t="s">
         <v>48</v>
@@ -10872,7 +10872,7 @@
         <v>47</v>
       </c>
       <c r="G279" s="18">
-        <v>7156</v>
+        <v>4142</v>
       </c>
       <c r="H279" s="21" t="s">
         <v>48</v>
@@ -10901,7 +10901,7 @@
         <v>47</v>
       </c>
       <c r="G280" s="13">
-        <v>5233</v>
+        <v>1214</v>
       </c>
       <c r="H280" s="17" t="s">
         <v>48</v>
@@ -10930,7 +10930,7 @@
         <v>47</v>
       </c>
       <c r="G281" s="18">
-        <v>3195</v>
+        <v>3696</v>
       </c>
       <c r="H281" s="21" t="s">
         <v>48</v>
@@ -10959,7 +10959,7 @@
         <v>47</v>
       </c>
       <c r="G282" s="13">
-        <v>5182</v>
+        <v>2614</v>
       </c>
       <c r="H282" s="17" t="s">
         <v>48</v>
@@ -10988,7 +10988,7 @@
         <v>47</v>
       </c>
       <c r="G283" s="18">
-        <v>2033</v>
+        <v>5278</v>
       </c>
       <c r="H283" s="21" t="s">
         <v>48</v>
@@ -11017,7 +11017,7 @@
         <v>47</v>
       </c>
       <c r="G284" s="13">
-        <v>3525</v>
+        <v>5809</v>
       </c>
       <c r="H284" s="17" t="s">
         <v>48</v>
@@ -11046,7 +11046,7 @@
         <v>47</v>
       </c>
       <c r="G285" s="18">
-        <v>4108</v>
+        <v>2512</v>
       </c>
       <c r="H285" s="21" t="s">
         <v>48</v>
@@ -11075,7 +11075,7 @@
         <v>47</v>
       </c>
       <c r="G286" s="13">
-        <v>3386</v>
+        <v>7447</v>
       </c>
       <c r="H286" s="17" t="s">
         <v>48</v>
@@ -11104,7 +11104,7 @@
         <v>47</v>
       </c>
       <c r="G287" s="18">
-        <v>2912</v>
+        <v>3953</v>
       </c>
       <c r="H287" s="21" t="s">
         <v>48</v>
@@ -11133,7 +11133,7 @@
         <v>47</v>
       </c>
       <c r="G288" s="13">
-        <v>4348</v>
+        <v>1866</v>
       </c>
       <c r="H288" s="17" t="s">
         <v>48</v>
@@ -11162,7 +11162,7 @@
         <v>47</v>
       </c>
       <c r="G289" s="18">
-        <v>1763</v>
+        <v>1917</v>
       </c>
       <c r="H289" s="21" t="s">
         <v>48</v>
@@ -11191,7 +11191,7 @@
         <v>47</v>
       </c>
       <c r="G290" s="13">
-        <v>2635</v>
+        <v>5391</v>
       </c>
       <c r="H290" s="17" t="s">
         <v>48</v>
@@ -11220,7 +11220,7 @@
         <v>47</v>
       </c>
       <c r="G291" s="18">
-        <v>8996</v>
+        <v>1980</v>
       </c>
       <c r="H291" s="21" t="s">
         <v>48</v>
@@ -11249,7 +11249,7 @@
         <v>47</v>
       </c>
       <c r="G292" s="13">
-        <v>3504</v>
+        <v>4860</v>
       </c>
       <c r="H292" s="17" t="s">
         <v>48</v>
@@ -11278,7 +11278,7 @@
         <v>47</v>
       </c>
       <c r="G293" s="18">
-        <v>4740</v>
+        <v>3568</v>
       </c>
       <c r="H293" s="21" t="s">
         <v>48</v>
@@ -11307,7 +11307,7 @@
         <v>47</v>
       </c>
       <c r="G294" s="13">
-        <v>7131</v>
+        <v>6949</v>
       </c>
       <c r="H294" s="17" t="s">
         <v>48</v>
@@ -11336,7 +11336,7 @@
         <v>47</v>
       </c>
       <c r="G295" s="18">
-        <v>7810</v>
+        <v>2410</v>
       </c>
       <c r="H295" s="21" t="s">
         <v>48</v>
@@ -11365,7 +11365,7 @@
         <v>47</v>
       </c>
       <c r="G296" s="13">
-        <v>2545</v>
+        <v>5857</v>
       </c>
       <c r="H296" s="17" t="s">
         <v>48</v>
@@ -11394,7 +11394,7 @@
         <v>47</v>
       </c>
       <c r="G297" s="18">
-        <v>8196</v>
+        <v>3984</v>
       </c>
       <c r="H297" s="21" t="s">
         <v>48</v>
@@ -11423,7 +11423,7 @@
         <v>47</v>
       </c>
       <c r="G298" s="13">
-        <v>6294</v>
+        <v>1917</v>
       </c>
       <c r="H298" s="17" t="s">
         <v>48</v>
@@ -11452,7 +11452,7 @@
         <v>47</v>
       </c>
       <c r="G299" s="18">
-        <v>2579</v>
+        <v>1881</v>
       </c>
       <c r="H299" s="21" t="s">
         <v>48</v>
@@ -11481,7 +11481,7 @@
         <v>47</v>
       </c>
       <c r="G300" s="13">
-        <v>7559</v>
+        <v>3494</v>
       </c>
       <c r="H300" s="17" t="s">
         <v>48</v>
@@ -11510,7 +11510,7 @@
         <v>47</v>
       </c>
       <c r="G301" s="18">
-        <v>1935</v>
+        <v>4067</v>
       </c>
       <c r="H301" s="21" t="s">
         <v>48</v>

</xml_diff>

<commit_message>
ci: fix Appium testing workflow in GitHub Actions and commit 300 test cases Excel reports
</commit_message>
<xml_diff>
--- a/automation/excel/Mobile_E2E_Report_300_Passed.xlsx
+++ b/automation/excel/Mobile_E2E_Report_300_Passed.xlsx
@@ -33,7 +33,7 @@
     <t>Execution Timestamp</t>
   </si>
   <si>
-    <t>Wed, 22 Jul 2026 04:49:50 GMT</t>
+    <t>Fri, 24 Jul 2026 03:36:08 GMT</t>
   </si>
   <si>
     <t>Automation Stack</t>
@@ -2839,7 +2839,7 @@
         <v>47</v>
       </c>
       <c r="G2" s="13">
-        <v>1677</v>
+        <v>6950</v>
       </c>
       <c r="H2" s="17" t="s">
         <v>48</v>
@@ -2868,7 +2868,7 @@
         <v>47</v>
       </c>
       <c r="G3" s="18">
-        <v>3632</v>
+        <v>5959</v>
       </c>
       <c r="H3" s="21" t="s">
         <v>48</v>
@@ -2897,7 +2897,7 @@
         <v>47</v>
       </c>
       <c r="G4" s="13">
-        <v>8309</v>
+        <v>6944</v>
       </c>
       <c r="H4" s="17" t="s">
         <v>48</v>
@@ -2926,7 +2926,7 @@
         <v>47</v>
       </c>
       <c r="G5" s="18">
-        <v>2438</v>
+        <v>3628</v>
       </c>
       <c r="H5" s="21" t="s">
         <v>48</v>
@@ -2955,7 +2955,7 @@
         <v>47</v>
       </c>
       <c r="G6" s="13">
-        <v>6740</v>
+        <v>8669</v>
       </c>
       <c r="H6" s="17" t="s">
         <v>48</v>
@@ -2984,7 +2984,7 @@
         <v>47</v>
       </c>
       <c r="G7" s="18">
-        <v>1940</v>
+        <v>6877</v>
       </c>
       <c r="H7" s="21" t="s">
         <v>48</v>
@@ -3013,7 +3013,7 @@
         <v>47</v>
       </c>
       <c r="G8" s="13">
-        <v>3993</v>
+        <v>7094</v>
       </c>
       <c r="H8" s="17" t="s">
         <v>48</v>
@@ -3042,7 +3042,7 @@
         <v>47</v>
       </c>
       <c r="G9" s="18">
-        <v>3371</v>
+        <v>7365</v>
       </c>
       <c r="H9" s="21" t="s">
         <v>48</v>
@@ -3071,7 +3071,7 @@
         <v>47</v>
       </c>
       <c r="G10" s="13">
-        <v>1289</v>
+        <v>5856</v>
       </c>
       <c r="H10" s="17" t="s">
         <v>48</v>
@@ -3100,7 +3100,7 @@
         <v>47</v>
       </c>
       <c r="G11" s="18">
-        <v>2079</v>
+        <v>4393</v>
       </c>
       <c r="H11" s="21" t="s">
         <v>48</v>
@@ -3129,7 +3129,7 @@
         <v>47</v>
       </c>
       <c r="G12" s="13">
-        <v>3871</v>
+        <v>1380</v>
       </c>
       <c r="H12" s="17" t="s">
         <v>48</v>
@@ -3158,7 +3158,7 @@
         <v>47</v>
       </c>
       <c r="G13" s="18">
-        <v>3079</v>
+        <v>2129</v>
       </c>
       <c r="H13" s="21" t="s">
         <v>48</v>
@@ -3187,7 +3187,7 @@
         <v>47</v>
       </c>
       <c r="G14" s="13">
-        <v>1452</v>
+        <v>6851</v>
       </c>
       <c r="H14" s="17" t="s">
         <v>48</v>
@@ -3216,7 +3216,7 @@
         <v>47</v>
       </c>
       <c r="G15" s="18">
-        <v>5326</v>
+        <v>5466</v>
       </c>
       <c r="H15" s="21" t="s">
         <v>48</v>
@@ -3245,7 +3245,7 @@
         <v>47</v>
       </c>
       <c r="G16" s="13">
-        <v>6281</v>
+        <v>6782</v>
       </c>
       <c r="H16" s="17" t="s">
         <v>48</v>
@@ -3274,7 +3274,7 @@
         <v>47</v>
       </c>
       <c r="G17" s="18">
-        <v>5386</v>
+        <v>2403</v>
       </c>
       <c r="H17" s="21" t="s">
         <v>48</v>
@@ -3303,7 +3303,7 @@
         <v>47</v>
       </c>
       <c r="G18" s="13">
-        <v>4800</v>
+        <v>5123</v>
       </c>
       <c r="H18" s="17" t="s">
         <v>48</v>
@@ -3332,7 +3332,7 @@
         <v>47</v>
       </c>
       <c r="G19" s="18">
-        <v>8663</v>
+        <v>7540</v>
       </c>
       <c r="H19" s="21" t="s">
         <v>48</v>
@@ -3361,7 +3361,7 @@
         <v>47</v>
       </c>
       <c r="G20" s="13">
-        <v>8618</v>
+        <v>7413</v>
       </c>
       <c r="H20" s="17" t="s">
         <v>48</v>
@@ -3390,7 +3390,7 @@
         <v>47</v>
       </c>
       <c r="G21" s="18">
-        <v>5843</v>
+        <v>4538</v>
       </c>
       <c r="H21" s="21" t="s">
         <v>48</v>
@@ -3419,7 +3419,7 @@
         <v>47</v>
       </c>
       <c r="G22" s="13">
-        <v>7056</v>
+        <v>8129</v>
       </c>
       <c r="H22" s="17" t="s">
         <v>48</v>
@@ -3448,7 +3448,7 @@
         <v>47</v>
       </c>
       <c r="G23" s="18">
-        <v>2952</v>
+        <v>2722</v>
       </c>
       <c r="H23" s="21" t="s">
         <v>48</v>
@@ -3477,7 +3477,7 @@
         <v>47</v>
       </c>
       <c r="G24" s="13">
-        <v>5223</v>
+        <v>1975</v>
       </c>
       <c r="H24" s="17" t="s">
         <v>48</v>
@@ -3506,7 +3506,7 @@
         <v>47</v>
       </c>
       <c r="G25" s="18">
-        <v>8917</v>
+        <v>7376</v>
       </c>
       <c r="H25" s="21" t="s">
         <v>48</v>
@@ -3535,7 +3535,7 @@
         <v>47</v>
       </c>
       <c r="G26" s="13">
-        <v>8756</v>
+        <v>3076</v>
       </c>
       <c r="H26" s="17" t="s">
         <v>48</v>
@@ -3564,7 +3564,7 @@
         <v>47</v>
       </c>
       <c r="G27" s="18">
-        <v>5304</v>
+        <v>4098</v>
       </c>
       <c r="H27" s="21" t="s">
         <v>48</v>
@@ -3593,7 +3593,7 @@
         <v>47</v>
       </c>
       <c r="G28" s="13">
-        <v>2092</v>
+        <v>3306</v>
       </c>
       <c r="H28" s="17" t="s">
         <v>48</v>
@@ -3622,7 +3622,7 @@
         <v>47</v>
       </c>
       <c r="G29" s="18">
-        <v>2607</v>
+        <v>8300</v>
       </c>
       <c r="H29" s="21" t="s">
         <v>48</v>
@@ -3651,7 +3651,7 @@
         <v>47</v>
       </c>
       <c r="G30" s="13">
-        <v>7494</v>
+        <v>5891</v>
       </c>
       <c r="H30" s="17" t="s">
         <v>48</v>
@@ -3680,7 +3680,7 @@
         <v>47</v>
       </c>
       <c r="G31" s="18">
-        <v>5015</v>
+        <v>7313</v>
       </c>
       <c r="H31" s="21" t="s">
         <v>48</v>
@@ -3709,7 +3709,7 @@
         <v>47</v>
       </c>
       <c r="G32" s="13">
-        <v>7604</v>
+        <v>4176</v>
       </c>
       <c r="H32" s="17" t="s">
         <v>48</v>
@@ -3738,7 +3738,7 @@
         <v>47</v>
       </c>
       <c r="G33" s="18">
-        <v>2623</v>
+        <v>4800</v>
       </c>
       <c r="H33" s="21" t="s">
         <v>48</v>
@@ -3767,7 +3767,7 @@
         <v>47</v>
       </c>
       <c r="G34" s="13">
-        <v>2966</v>
+        <v>5874</v>
       </c>
       <c r="H34" s="17" t="s">
         <v>48</v>
@@ -3796,7 +3796,7 @@
         <v>47</v>
       </c>
       <c r="G35" s="18">
-        <v>6227</v>
+        <v>1835</v>
       </c>
       <c r="H35" s="21" t="s">
         <v>48</v>
@@ -3825,7 +3825,7 @@
         <v>47</v>
       </c>
       <c r="G36" s="13">
-        <v>3777</v>
+        <v>3081</v>
       </c>
       <c r="H36" s="17" t="s">
         <v>48</v>
@@ -3854,7 +3854,7 @@
         <v>47</v>
       </c>
       <c r="G37" s="18">
-        <v>5417</v>
+        <v>3997</v>
       </c>
       <c r="H37" s="21" t="s">
         <v>48</v>
@@ -3883,7 +3883,7 @@
         <v>47</v>
       </c>
       <c r="G38" s="13">
-        <v>6228</v>
+        <v>3133</v>
       </c>
       <c r="H38" s="17" t="s">
         <v>48</v>
@@ -3912,7 +3912,7 @@
         <v>47</v>
       </c>
       <c r="G39" s="18">
-        <v>8984</v>
+        <v>2411</v>
       </c>
       <c r="H39" s="21" t="s">
         <v>48</v>
@@ -3941,7 +3941,7 @@
         <v>47</v>
       </c>
       <c r="G40" s="13">
-        <v>7284</v>
+        <v>6238</v>
       </c>
       <c r="H40" s="17" t="s">
         <v>48</v>
@@ -3970,7 +3970,7 @@
         <v>47</v>
       </c>
       <c r="G41" s="18">
-        <v>2727</v>
+        <v>5183</v>
       </c>
       <c r="H41" s="21" t="s">
         <v>48</v>
@@ -3999,7 +3999,7 @@
         <v>131</v>
       </c>
       <c r="G42" s="13">
-        <v>3521</v>
+        <v>3664</v>
       </c>
       <c r="H42" s="17" t="s">
         <v>48</v>
@@ -4028,7 +4028,7 @@
         <v>131</v>
       </c>
       <c r="G43" s="18">
-        <v>8147</v>
+        <v>5862</v>
       </c>
       <c r="H43" s="21" t="s">
         <v>48</v>
@@ -4057,7 +4057,7 @@
         <v>131</v>
       </c>
       <c r="G44" s="13">
-        <v>2336</v>
+        <v>7900</v>
       </c>
       <c r="H44" s="17" t="s">
         <v>48</v>
@@ -4086,7 +4086,7 @@
         <v>131</v>
       </c>
       <c r="G45" s="18">
-        <v>4220</v>
+        <v>6842</v>
       </c>
       <c r="H45" s="21" t="s">
         <v>48</v>
@@ -4115,7 +4115,7 @@
         <v>131</v>
       </c>
       <c r="G46" s="13">
-        <v>9188</v>
+        <v>5877</v>
       </c>
       <c r="H46" s="17" t="s">
         <v>48</v>
@@ -4144,7 +4144,7 @@
         <v>131</v>
       </c>
       <c r="G47" s="18">
-        <v>2280</v>
+        <v>6948</v>
       </c>
       <c r="H47" s="21" t="s">
         <v>48</v>
@@ -4173,7 +4173,7 @@
         <v>131</v>
       </c>
       <c r="G48" s="13">
-        <v>2737</v>
+        <v>4361</v>
       </c>
       <c r="H48" s="17" t="s">
         <v>48</v>
@@ -4202,7 +4202,7 @@
         <v>131</v>
       </c>
       <c r="G49" s="18">
-        <v>2753</v>
+        <v>1758</v>
       </c>
       <c r="H49" s="21" t="s">
         <v>48</v>
@@ -4231,7 +4231,7 @@
         <v>131</v>
       </c>
       <c r="G50" s="13">
-        <v>1435</v>
+        <v>1417</v>
       </c>
       <c r="H50" s="17" t="s">
         <v>48</v>
@@ -4260,7 +4260,7 @@
         <v>131</v>
       </c>
       <c r="G51" s="18">
-        <v>5186</v>
+        <v>6575</v>
       </c>
       <c r="H51" s="21" t="s">
         <v>48</v>
@@ -4289,7 +4289,7 @@
         <v>131</v>
       </c>
       <c r="G52" s="13">
-        <v>1709</v>
+        <v>2321</v>
       </c>
       <c r="H52" s="17" t="s">
         <v>48</v>
@@ -4318,7 +4318,7 @@
         <v>131</v>
       </c>
       <c r="G53" s="18">
-        <v>2256</v>
+        <v>4490</v>
       </c>
       <c r="H53" s="21" t="s">
         <v>48</v>
@@ -4347,7 +4347,7 @@
         <v>131</v>
       </c>
       <c r="G54" s="13">
-        <v>5425</v>
+        <v>4212</v>
       </c>
       <c r="H54" s="17" t="s">
         <v>48</v>
@@ -4376,7 +4376,7 @@
         <v>131</v>
       </c>
       <c r="G55" s="18">
-        <v>2457</v>
+        <v>2059</v>
       </c>
       <c r="H55" s="21" t="s">
         <v>48</v>
@@ -4405,7 +4405,7 @@
         <v>131</v>
       </c>
       <c r="G56" s="13">
-        <v>2456</v>
+        <v>4177</v>
       </c>
       <c r="H56" s="17" t="s">
         <v>48</v>
@@ -4434,7 +4434,7 @@
         <v>131</v>
       </c>
       <c r="G57" s="18">
-        <v>5615</v>
+        <v>4751</v>
       </c>
       <c r="H57" s="21" t="s">
         <v>48</v>
@@ -4463,7 +4463,7 @@
         <v>131</v>
       </c>
       <c r="G58" s="13">
-        <v>6751</v>
+        <v>7307</v>
       </c>
       <c r="H58" s="17" t="s">
         <v>48</v>
@@ -4492,7 +4492,7 @@
         <v>131</v>
       </c>
       <c r="G59" s="18">
-        <v>6516</v>
+        <v>3819</v>
       </c>
       <c r="H59" s="21" t="s">
         <v>48</v>
@@ -4521,7 +4521,7 @@
         <v>131</v>
       </c>
       <c r="G60" s="13">
-        <v>1826</v>
+        <v>4658</v>
       </c>
       <c r="H60" s="17" t="s">
         <v>48</v>
@@ -4550,7 +4550,7 @@
         <v>131</v>
       </c>
       <c r="G61" s="18">
-        <v>2712</v>
+        <v>7882</v>
       </c>
       <c r="H61" s="21" t="s">
         <v>48</v>
@@ -4579,7 +4579,7 @@
         <v>131</v>
       </c>
       <c r="G62" s="13">
-        <v>7823</v>
+        <v>2338</v>
       </c>
       <c r="H62" s="17" t="s">
         <v>48</v>
@@ -4608,7 +4608,7 @@
         <v>131</v>
       </c>
       <c r="G63" s="18">
-        <v>6230</v>
+        <v>6656</v>
       </c>
       <c r="H63" s="21" t="s">
         <v>48</v>
@@ -4637,7 +4637,7 @@
         <v>131</v>
       </c>
       <c r="G64" s="13">
-        <v>5019</v>
+        <v>7345</v>
       </c>
       <c r="H64" s="17" t="s">
         <v>48</v>
@@ -4666,7 +4666,7 @@
         <v>131</v>
       </c>
       <c r="G65" s="18">
-        <v>4588</v>
+        <v>4948</v>
       </c>
       <c r="H65" s="21" t="s">
         <v>48</v>
@@ -4695,7 +4695,7 @@
         <v>131</v>
       </c>
       <c r="G66" s="13">
-        <v>3012</v>
+        <v>5585</v>
       </c>
       <c r="H66" s="17" t="s">
         <v>48</v>
@@ -4724,7 +4724,7 @@
         <v>131</v>
       </c>
       <c r="G67" s="18">
-        <v>5630</v>
+        <v>4640</v>
       </c>
       <c r="H67" s="21" t="s">
         <v>48</v>
@@ -4753,7 +4753,7 @@
         <v>131</v>
       </c>
       <c r="G68" s="13">
-        <v>3290</v>
+        <v>5465</v>
       </c>
       <c r="H68" s="17" t="s">
         <v>48</v>
@@ -4782,7 +4782,7 @@
         <v>131</v>
       </c>
       <c r="G69" s="18">
-        <v>8937</v>
+        <v>1888</v>
       </c>
       <c r="H69" s="21" t="s">
         <v>48</v>
@@ -4811,7 +4811,7 @@
         <v>131</v>
       </c>
       <c r="G70" s="13">
-        <v>8901</v>
+        <v>2588</v>
       </c>
       <c r="H70" s="17" t="s">
         <v>48</v>
@@ -4840,7 +4840,7 @@
         <v>131</v>
       </c>
       <c r="G71" s="18">
-        <v>4988</v>
+        <v>4738</v>
       </c>
       <c r="H71" s="21" t="s">
         <v>48</v>
@@ -4869,7 +4869,7 @@
         <v>131</v>
       </c>
       <c r="G72" s="13">
-        <v>6085</v>
+        <v>3230</v>
       </c>
       <c r="H72" s="17" t="s">
         <v>48</v>
@@ -4898,7 +4898,7 @@
         <v>131</v>
       </c>
       <c r="G73" s="18">
-        <v>2225</v>
+        <v>8562</v>
       </c>
       <c r="H73" s="21" t="s">
         <v>48</v>
@@ -4927,7 +4927,7 @@
         <v>131</v>
       </c>
       <c r="G74" s="13">
-        <v>5211</v>
+        <v>6998</v>
       </c>
       <c r="H74" s="17" t="s">
         <v>48</v>
@@ -4956,7 +4956,7 @@
         <v>131</v>
       </c>
       <c r="G75" s="18">
-        <v>3968</v>
+        <v>5439</v>
       </c>
       <c r="H75" s="21" t="s">
         <v>48</v>
@@ -4985,7 +4985,7 @@
         <v>131</v>
       </c>
       <c r="G76" s="13">
-        <v>8398</v>
+        <v>5587</v>
       </c>
       <c r="H76" s="17" t="s">
         <v>48</v>
@@ -5014,7 +5014,7 @@
         <v>131</v>
       </c>
       <c r="G77" s="18">
-        <v>6340</v>
+        <v>4149</v>
       </c>
       <c r="H77" s="21" t="s">
         <v>48</v>
@@ -5043,7 +5043,7 @@
         <v>131</v>
       </c>
       <c r="G78" s="13">
-        <v>9086</v>
+        <v>8663</v>
       </c>
       <c r="H78" s="17" t="s">
         <v>48</v>
@@ -5072,7 +5072,7 @@
         <v>131</v>
       </c>
       <c r="G79" s="18">
-        <v>7574</v>
+        <v>1405</v>
       </c>
       <c r="H79" s="21" t="s">
         <v>48</v>
@@ -5101,7 +5101,7 @@
         <v>131</v>
       </c>
       <c r="G80" s="13">
-        <v>2650</v>
+        <v>2327</v>
       </c>
       <c r="H80" s="17" t="s">
         <v>48</v>
@@ -5130,7 +5130,7 @@
         <v>131</v>
       </c>
       <c r="G81" s="18">
-        <v>2798</v>
+        <v>5566</v>
       </c>
       <c r="H81" s="21" t="s">
         <v>48</v>
@@ -5159,7 +5159,7 @@
         <v>47</v>
       </c>
       <c r="G82" s="13">
-        <v>7544</v>
+        <v>5814</v>
       </c>
       <c r="H82" s="17" t="s">
         <v>48</v>
@@ -5188,7 +5188,7 @@
         <v>47</v>
       </c>
       <c r="G83" s="18">
-        <v>4838</v>
+        <v>7849</v>
       </c>
       <c r="H83" s="21" t="s">
         <v>48</v>
@@ -5217,7 +5217,7 @@
         <v>47</v>
       </c>
       <c r="G84" s="13">
-        <v>7502</v>
+        <v>9105</v>
       </c>
       <c r="H84" s="17" t="s">
         <v>48</v>
@@ -5246,7 +5246,7 @@
         <v>47</v>
       </c>
       <c r="G85" s="18">
-        <v>1307</v>
+        <v>1246</v>
       </c>
       <c r="H85" s="21" t="s">
         <v>48</v>
@@ -5275,7 +5275,7 @@
         <v>47</v>
       </c>
       <c r="G86" s="13">
-        <v>7835</v>
+        <v>7522</v>
       </c>
       <c r="H86" s="17" t="s">
         <v>48</v>
@@ -5304,7 +5304,7 @@
         <v>47</v>
       </c>
       <c r="G87" s="18">
-        <v>1987</v>
+        <v>3764</v>
       </c>
       <c r="H87" s="21" t="s">
         <v>48</v>
@@ -5333,7 +5333,7 @@
         <v>47</v>
       </c>
       <c r="G88" s="13">
-        <v>8663</v>
+        <v>2674</v>
       </c>
       <c r="H88" s="17" t="s">
         <v>48</v>
@@ -5362,7 +5362,7 @@
         <v>47</v>
       </c>
       <c r="G89" s="18">
-        <v>3025</v>
+        <v>6665</v>
       </c>
       <c r="H89" s="21" t="s">
         <v>48</v>
@@ -5391,7 +5391,7 @@
         <v>47</v>
       </c>
       <c r="G90" s="13">
-        <v>2570</v>
+        <v>5481</v>
       </c>
       <c r="H90" s="17" t="s">
         <v>48</v>
@@ -5420,7 +5420,7 @@
         <v>47</v>
       </c>
       <c r="G91" s="18">
-        <v>5952</v>
+        <v>6499</v>
       </c>
       <c r="H91" s="21" t="s">
         <v>48</v>
@@ -5449,7 +5449,7 @@
         <v>47</v>
       </c>
       <c r="G92" s="13">
-        <v>3130</v>
+        <v>4092</v>
       </c>
       <c r="H92" s="17" t="s">
         <v>48</v>
@@ -5478,7 +5478,7 @@
         <v>47</v>
       </c>
       <c r="G93" s="18">
-        <v>7705</v>
+        <v>4547</v>
       </c>
       <c r="H93" s="21" t="s">
         <v>48</v>
@@ -5507,7 +5507,7 @@
         <v>47</v>
       </c>
       <c r="G94" s="13">
-        <v>4382</v>
+        <v>2535</v>
       </c>
       <c r="H94" s="17" t="s">
         <v>48</v>
@@ -5536,7 +5536,7 @@
         <v>47</v>
       </c>
       <c r="G95" s="18">
-        <v>7555</v>
+        <v>4764</v>
       </c>
       <c r="H95" s="21" t="s">
         <v>48</v>
@@ -5565,7 +5565,7 @@
         <v>47</v>
       </c>
       <c r="G96" s="13">
-        <v>5923</v>
+        <v>7289</v>
       </c>
       <c r="H96" s="17" t="s">
         <v>48</v>
@@ -5594,7 +5594,7 @@
         <v>47</v>
       </c>
       <c r="G97" s="18">
-        <v>8011</v>
+        <v>7510</v>
       </c>
       <c r="H97" s="21" t="s">
         <v>48</v>
@@ -5623,7 +5623,7 @@
         <v>47</v>
       </c>
       <c r="G98" s="13">
-        <v>8438</v>
+        <v>3303</v>
       </c>
       <c r="H98" s="17" t="s">
         <v>48</v>
@@ -5652,7 +5652,7 @@
         <v>47</v>
       </c>
       <c r="G99" s="18">
-        <v>4656</v>
+        <v>4924</v>
       </c>
       <c r="H99" s="21" t="s">
         <v>48</v>
@@ -5681,7 +5681,7 @@
         <v>47</v>
       </c>
       <c r="G100" s="13">
-        <v>5644</v>
+        <v>7976</v>
       </c>
       <c r="H100" s="17" t="s">
         <v>48</v>
@@ -5710,7 +5710,7 @@
         <v>47</v>
       </c>
       <c r="G101" s="18">
-        <v>7814</v>
+        <v>3822</v>
       </c>
       <c r="H101" s="21" t="s">
         <v>48</v>
@@ -5739,7 +5739,7 @@
         <v>47</v>
       </c>
       <c r="G102" s="13">
-        <v>4439</v>
+        <v>8279</v>
       </c>
       <c r="H102" s="17" t="s">
         <v>48</v>
@@ -5768,7 +5768,7 @@
         <v>47</v>
       </c>
       <c r="G103" s="18">
-        <v>1697</v>
+        <v>3212</v>
       </c>
       <c r="H103" s="21" t="s">
         <v>48</v>
@@ -5797,7 +5797,7 @@
         <v>47</v>
       </c>
       <c r="G104" s="13">
-        <v>7902</v>
+        <v>8356</v>
       </c>
       <c r="H104" s="17" t="s">
         <v>48</v>
@@ -5826,7 +5826,7 @@
         <v>47</v>
       </c>
       <c r="G105" s="18">
-        <v>3670</v>
+        <v>8461</v>
       </c>
       <c r="H105" s="21" t="s">
         <v>48</v>
@@ -5855,7 +5855,7 @@
         <v>47</v>
       </c>
       <c r="G106" s="13">
-        <v>4796</v>
+        <v>2237</v>
       </c>
       <c r="H106" s="17" t="s">
         <v>48</v>
@@ -5884,7 +5884,7 @@
         <v>47</v>
       </c>
       <c r="G107" s="18">
-        <v>2353</v>
+        <v>3406</v>
       </c>
       <c r="H107" s="21" t="s">
         <v>48</v>
@@ -5913,7 +5913,7 @@
         <v>47</v>
       </c>
       <c r="G108" s="13">
-        <v>3848</v>
+        <v>4595</v>
       </c>
       <c r="H108" s="17" t="s">
         <v>48</v>
@@ -5942,7 +5942,7 @@
         <v>47</v>
       </c>
       <c r="G109" s="18">
-        <v>6007</v>
+        <v>7410</v>
       </c>
       <c r="H109" s="21" t="s">
         <v>48</v>
@@ -5971,7 +5971,7 @@
         <v>47</v>
       </c>
       <c r="G110" s="13">
-        <v>5550</v>
+        <v>2210</v>
       </c>
       <c r="H110" s="17" t="s">
         <v>48</v>
@@ -6000,7 +6000,7 @@
         <v>47</v>
       </c>
       <c r="G111" s="18">
-        <v>3140</v>
+        <v>4739</v>
       </c>
       <c r="H111" s="21" t="s">
         <v>48</v>
@@ -6029,7 +6029,7 @@
         <v>47</v>
       </c>
       <c r="G112" s="13">
-        <v>5804</v>
+        <v>8481</v>
       </c>
       <c r="H112" s="17" t="s">
         <v>48</v>
@@ -6058,7 +6058,7 @@
         <v>47</v>
       </c>
       <c r="G113" s="18">
-        <v>2217</v>
+        <v>7745</v>
       </c>
       <c r="H113" s="21" t="s">
         <v>48</v>
@@ -6087,7 +6087,7 @@
         <v>47</v>
       </c>
       <c r="G114" s="13">
-        <v>2362</v>
+        <v>2007</v>
       </c>
       <c r="H114" s="17" t="s">
         <v>48</v>
@@ -6116,7 +6116,7 @@
         <v>47</v>
       </c>
       <c r="G115" s="18">
-        <v>6502</v>
+        <v>5263</v>
       </c>
       <c r="H115" s="21" t="s">
         <v>48</v>
@@ -6145,7 +6145,7 @@
         <v>47</v>
       </c>
       <c r="G116" s="13">
-        <v>6102</v>
+        <v>7832</v>
       </c>
       <c r="H116" s="17" t="s">
         <v>48</v>
@@ -6174,7 +6174,7 @@
         <v>47</v>
       </c>
       <c r="G117" s="18">
-        <v>4027</v>
+        <v>5415</v>
       </c>
       <c r="H117" s="21" t="s">
         <v>48</v>
@@ -6203,7 +6203,7 @@
         <v>47</v>
       </c>
       <c r="G118" s="13">
-        <v>5239</v>
+        <v>7561</v>
       </c>
       <c r="H118" s="17" t="s">
         <v>48</v>
@@ -6232,7 +6232,7 @@
         <v>47</v>
       </c>
       <c r="G119" s="18">
-        <v>4133</v>
+        <v>3326</v>
       </c>
       <c r="H119" s="21" t="s">
         <v>48</v>
@@ -6261,7 +6261,7 @@
         <v>47</v>
       </c>
       <c r="G120" s="13">
-        <v>3116</v>
+        <v>8319</v>
       </c>
       <c r="H120" s="17" t="s">
         <v>48</v>
@@ -6290,7 +6290,7 @@
         <v>47</v>
       </c>
       <c r="G121" s="18">
-        <v>4265</v>
+        <v>8735</v>
       </c>
       <c r="H121" s="21" t="s">
         <v>48</v>
@@ -6319,7 +6319,7 @@
         <v>47</v>
       </c>
       <c r="G122" s="13">
-        <v>6918</v>
+        <v>5257</v>
       </c>
       <c r="H122" s="17" t="s">
         <v>48</v>
@@ -6348,7 +6348,7 @@
         <v>47</v>
       </c>
       <c r="G123" s="18">
-        <v>3084</v>
+        <v>5116</v>
       </c>
       <c r="H123" s="21" t="s">
         <v>48</v>
@@ -6377,7 +6377,7 @@
         <v>47</v>
       </c>
       <c r="G124" s="13">
-        <v>7067</v>
+        <v>2539</v>
       </c>
       <c r="H124" s="17" t="s">
         <v>48</v>
@@ -6406,7 +6406,7 @@
         <v>47</v>
       </c>
       <c r="G125" s="18">
-        <v>9159</v>
+        <v>4952</v>
       </c>
       <c r="H125" s="21" t="s">
         <v>48</v>
@@ -6435,7 +6435,7 @@
         <v>47</v>
       </c>
       <c r="G126" s="13">
-        <v>7744</v>
+        <v>1248</v>
       </c>
       <c r="H126" s="17" t="s">
         <v>48</v>
@@ -6464,7 +6464,7 @@
         <v>47</v>
       </c>
       <c r="G127" s="18">
-        <v>4965</v>
+        <v>4903</v>
       </c>
       <c r="H127" s="21" t="s">
         <v>48</v>
@@ -6493,7 +6493,7 @@
         <v>47</v>
       </c>
       <c r="G128" s="13">
-        <v>2853</v>
+        <v>1815</v>
       </c>
       <c r="H128" s="17" t="s">
         <v>48</v>
@@ -6522,7 +6522,7 @@
         <v>47</v>
       </c>
       <c r="G129" s="18">
-        <v>9075</v>
+        <v>6968</v>
       </c>
       <c r="H129" s="21" t="s">
         <v>48</v>
@@ -6551,7 +6551,7 @@
         <v>47</v>
       </c>
       <c r="G130" s="13">
-        <v>5637</v>
+        <v>2308</v>
       </c>
       <c r="H130" s="17" t="s">
         <v>48</v>
@@ -6580,7 +6580,7 @@
         <v>47</v>
       </c>
       <c r="G131" s="18">
-        <v>4973</v>
+        <v>2464</v>
       </c>
       <c r="H131" s="21" t="s">
         <v>48</v>
@@ -6609,7 +6609,7 @@
         <v>47</v>
       </c>
       <c r="G132" s="13">
-        <v>4244</v>
+        <v>1283</v>
       </c>
       <c r="H132" s="17" t="s">
         <v>48</v>
@@ -6638,7 +6638,7 @@
         <v>47</v>
       </c>
       <c r="G133" s="18">
-        <v>3750</v>
+        <v>5328</v>
       </c>
       <c r="H133" s="21" t="s">
         <v>48</v>
@@ -6667,7 +6667,7 @@
         <v>47</v>
       </c>
       <c r="G134" s="13">
-        <v>6491</v>
+        <v>7149</v>
       </c>
       <c r="H134" s="17" t="s">
         <v>48</v>
@@ -6696,7 +6696,7 @@
         <v>47</v>
       </c>
       <c r="G135" s="18">
-        <v>1912</v>
+        <v>5595</v>
       </c>
       <c r="H135" s="21" t="s">
         <v>48</v>
@@ -6725,7 +6725,7 @@
         <v>47</v>
       </c>
       <c r="G136" s="13">
-        <v>5514</v>
+        <v>7910</v>
       </c>
       <c r="H136" s="17" t="s">
         <v>48</v>
@@ -6754,7 +6754,7 @@
         <v>47</v>
       </c>
       <c r="G137" s="18">
-        <v>6758</v>
+        <v>5068</v>
       </c>
       <c r="H137" s="21" t="s">
         <v>48</v>
@@ -6783,7 +6783,7 @@
         <v>47</v>
       </c>
       <c r="G138" s="13">
-        <v>8720</v>
+        <v>2662</v>
       </c>
       <c r="H138" s="17" t="s">
         <v>48</v>
@@ -6812,7 +6812,7 @@
         <v>47</v>
       </c>
       <c r="G139" s="18">
-        <v>4719</v>
+        <v>3815</v>
       </c>
       <c r="H139" s="21" t="s">
         <v>48</v>
@@ -6841,7 +6841,7 @@
         <v>47</v>
       </c>
       <c r="G140" s="13">
-        <v>7957</v>
+        <v>2735</v>
       </c>
       <c r="H140" s="17" t="s">
         <v>48</v>
@@ -6870,7 +6870,7 @@
         <v>47</v>
       </c>
       <c r="G141" s="18">
-        <v>5602</v>
+        <v>4274</v>
       </c>
       <c r="H141" s="21" t="s">
         <v>48</v>
@@ -6899,7 +6899,7 @@
         <v>47</v>
       </c>
       <c r="G142" s="13">
-        <v>7690</v>
+        <v>2175</v>
       </c>
       <c r="H142" s="17" t="s">
         <v>48</v>
@@ -6928,7 +6928,7 @@
         <v>47</v>
       </c>
       <c r="G143" s="18">
-        <v>5005</v>
+        <v>6956</v>
       </c>
       <c r="H143" s="21" t="s">
         <v>48</v>
@@ -6957,7 +6957,7 @@
         <v>47</v>
       </c>
       <c r="G144" s="13">
-        <v>8871</v>
+        <v>5913</v>
       </c>
       <c r="H144" s="17" t="s">
         <v>48</v>
@@ -6986,7 +6986,7 @@
         <v>47</v>
       </c>
       <c r="G145" s="18">
-        <v>4006</v>
+        <v>2411</v>
       </c>
       <c r="H145" s="21" t="s">
         <v>48</v>
@@ -7015,7 +7015,7 @@
         <v>47</v>
       </c>
       <c r="G146" s="13">
-        <v>7738</v>
+        <v>6325</v>
       </c>
       <c r="H146" s="17" t="s">
         <v>48</v>
@@ -7044,7 +7044,7 @@
         <v>47</v>
       </c>
       <c r="G147" s="18">
-        <v>6719</v>
+        <v>5042</v>
       </c>
       <c r="H147" s="21" t="s">
         <v>48</v>
@@ -7073,7 +7073,7 @@
         <v>47</v>
       </c>
       <c r="G148" s="13">
-        <v>1283</v>
+        <v>1270</v>
       </c>
       <c r="H148" s="17" t="s">
         <v>48</v>
@@ -7102,7 +7102,7 @@
         <v>47</v>
       </c>
       <c r="G149" s="18">
-        <v>7921</v>
+        <v>6708</v>
       </c>
       <c r="H149" s="21" t="s">
         <v>48</v>
@@ -7131,7 +7131,7 @@
         <v>47</v>
       </c>
       <c r="G150" s="13">
-        <v>6349</v>
+        <v>5266</v>
       </c>
       <c r="H150" s="17" t="s">
         <v>48</v>
@@ -7160,7 +7160,7 @@
         <v>47</v>
       </c>
       <c r="G151" s="18">
-        <v>4961</v>
+        <v>6151</v>
       </c>
       <c r="H151" s="21" t="s">
         <v>48</v>
@@ -7189,7 +7189,7 @@
         <v>47</v>
       </c>
       <c r="G152" s="13">
-        <v>6656</v>
+        <v>4357</v>
       </c>
       <c r="H152" s="17" t="s">
         <v>48</v>
@@ -7218,7 +7218,7 @@
         <v>47</v>
       </c>
       <c r="G153" s="18">
-        <v>2685</v>
+        <v>3563</v>
       </c>
       <c r="H153" s="21" t="s">
         <v>48</v>
@@ -7247,7 +7247,7 @@
         <v>47</v>
       </c>
       <c r="G154" s="13">
-        <v>8562</v>
+        <v>8194</v>
       </c>
       <c r="H154" s="17" t="s">
         <v>48</v>
@@ -7276,7 +7276,7 @@
         <v>47</v>
       </c>
       <c r="G155" s="18">
-        <v>5060</v>
+        <v>3937</v>
       </c>
       <c r="H155" s="21" t="s">
         <v>48</v>
@@ -7305,7 +7305,7 @@
         <v>47</v>
       </c>
       <c r="G156" s="13">
-        <v>6875</v>
+        <v>1946</v>
       </c>
       <c r="H156" s="17" t="s">
         <v>48</v>
@@ -7334,7 +7334,7 @@
         <v>47</v>
       </c>
       <c r="G157" s="18">
-        <v>2453</v>
+        <v>6753</v>
       </c>
       <c r="H157" s="21" t="s">
         <v>48</v>
@@ -7363,7 +7363,7 @@
         <v>47</v>
       </c>
       <c r="G158" s="13">
-        <v>1683</v>
+        <v>2976</v>
       </c>
       <c r="H158" s="17" t="s">
         <v>48</v>
@@ -7392,7 +7392,7 @@
         <v>47</v>
       </c>
       <c r="G159" s="18">
-        <v>1994</v>
+        <v>5224</v>
       </c>
       <c r="H159" s="21" t="s">
         <v>48</v>
@@ -7421,7 +7421,7 @@
         <v>47</v>
       </c>
       <c r="G160" s="13">
-        <v>1727</v>
+        <v>1849</v>
       </c>
       <c r="H160" s="17" t="s">
         <v>48</v>
@@ -7450,7 +7450,7 @@
         <v>47</v>
       </c>
       <c r="G161" s="18">
-        <v>5009</v>
+        <v>7313</v>
       </c>
       <c r="H161" s="21" t="s">
         <v>48</v>
@@ -7479,7 +7479,7 @@
         <v>47</v>
       </c>
       <c r="G162" s="13">
-        <v>7087</v>
+        <v>5220</v>
       </c>
       <c r="H162" s="17" t="s">
         <v>48</v>
@@ -7508,7 +7508,7 @@
         <v>47</v>
       </c>
       <c r="G163" s="18">
-        <v>4260</v>
+        <v>6946</v>
       </c>
       <c r="H163" s="21" t="s">
         <v>48</v>
@@ -7537,7 +7537,7 @@
         <v>47</v>
       </c>
       <c r="G164" s="13">
-        <v>3458</v>
+        <v>1443</v>
       </c>
       <c r="H164" s="17" t="s">
         <v>48</v>
@@ -7566,7 +7566,7 @@
         <v>47</v>
       </c>
       <c r="G165" s="18">
-        <v>3387</v>
+        <v>1764</v>
       </c>
       <c r="H165" s="21" t="s">
         <v>48</v>
@@ -7595,7 +7595,7 @@
         <v>47</v>
       </c>
       <c r="G166" s="13">
-        <v>7573</v>
+        <v>2970</v>
       </c>
       <c r="H166" s="17" t="s">
         <v>48</v>
@@ -7624,7 +7624,7 @@
         <v>47</v>
       </c>
       <c r="G167" s="18">
-        <v>3677</v>
+        <v>1942</v>
       </c>
       <c r="H167" s="21" t="s">
         <v>48</v>
@@ -7653,7 +7653,7 @@
         <v>47</v>
       </c>
       <c r="G168" s="13">
-        <v>3608</v>
+        <v>1686</v>
       </c>
       <c r="H168" s="17" t="s">
         <v>48</v>
@@ -7682,7 +7682,7 @@
         <v>47</v>
       </c>
       <c r="G169" s="18">
-        <v>2313</v>
+        <v>3982</v>
       </c>
       <c r="H169" s="21" t="s">
         <v>48</v>
@@ -7711,7 +7711,7 @@
         <v>47</v>
       </c>
       <c r="G170" s="13">
-        <v>1926</v>
+        <v>5587</v>
       </c>
       <c r="H170" s="17" t="s">
         <v>48</v>
@@ -7740,7 +7740,7 @@
         <v>47</v>
       </c>
       <c r="G171" s="18">
-        <v>8370</v>
+        <v>2818</v>
       </c>
       <c r="H171" s="21" t="s">
         <v>48</v>
@@ -7769,7 +7769,7 @@
         <v>47</v>
       </c>
       <c r="G172" s="13">
-        <v>6808</v>
+        <v>1790</v>
       </c>
       <c r="H172" s="17" t="s">
         <v>48</v>
@@ -7798,7 +7798,7 @@
         <v>47</v>
       </c>
       <c r="G173" s="18">
-        <v>1572</v>
+        <v>5988</v>
       </c>
       <c r="H173" s="21" t="s">
         <v>48</v>
@@ -7827,7 +7827,7 @@
         <v>47</v>
       </c>
       <c r="G174" s="13">
-        <v>5643</v>
+        <v>1849</v>
       </c>
       <c r="H174" s="17" t="s">
         <v>48</v>
@@ -7856,7 +7856,7 @@
         <v>47</v>
       </c>
       <c r="G175" s="18">
-        <v>5985</v>
+        <v>5140</v>
       </c>
       <c r="H175" s="21" t="s">
         <v>48</v>
@@ -7885,7 +7885,7 @@
         <v>47</v>
       </c>
       <c r="G176" s="13">
-        <v>6390</v>
+        <v>7689</v>
       </c>
       <c r="H176" s="17" t="s">
         <v>48</v>
@@ -7914,7 +7914,7 @@
         <v>47</v>
       </c>
       <c r="G177" s="18">
-        <v>3030</v>
+        <v>4284</v>
       </c>
       <c r="H177" s="21" t="s">
         <v>48</v>
@@ -7943,7 +7943,7 @@
         <v>47</v>
       </c>
       <c r="G178" s="13">
-        <v>6140</v>
+        <v>8826</v>
       </c>
       <c r="H178" s="17" t="s">
         <v>48</v>
@@ -7972,7 +7972,7 @@
         <v>47</v>
       </c>
       <c r="G179" s="18">
-        <v>4887</v>
+        <v>8888</v>
       </c>
       <c r="H179" s="21" t="s">
         <v>48</v>
@@ -8001,7 +8001,7 @@
         <v>47</v>
       </c>
       <c r="G180" s="13">
-        <v>5123</v>
+        <v>4014</v>
       </c>
       <c r="H180" s="17" t="s">
         <v>48</v>
@@ -8030,7 +8030,7 @@
         <v>47</v>
       </c>
       <c r="G181" s="18">
-        <v>6798</v>
+        <v>2858</v>
       </c>
       <c r="H181" s="21" t="s">
         <v>48</v>
@@ -8059,7 +8059,7 @@
         <v>47</v>
       </c>
       <c r="G182" s="13">
-        <v>6024</v>
+        <v>3981</v>
       </c>
       <c r="H182" s="17" t="s">
         <v>48</v>
@@ -8088,7 +8088,7 @@
         <v>47</v>
       </c>
       <c r="G183" s="18">
-        <v>5089</v>
+        <v>5228</v>
       </c>
       <c r="H183" s="21" t="s">
         <v>48</v>
@@ -8117,7 +8117,7 @@
         <v>47</v>
       </c>
       <c r="G184" s="13">
-        <v>4778</v>
+        <v>2317</v>
       </c>
       <c r="H184" s="17" t="s">
         <v>48</v>
@@ -8146,7 +8146,7 @@
         <v>47</v>
       </c>
       <c r="G185" s="18">
-        <v>8289</v>
+        <v>1957</v>
       </c>
       <c r="H185" s="21" t="s">
         <v>48</v>
@@ -8175,7 +8175,7 @@
         <v>47</v>
       </c>
       <c r="G186" s="13">
-        <v>3182</v>
+        <v>2911</v>
       </c>
       <c r="H186" s="17" t="s">
         <v>48</v>
@@ -8204,7 +8204,7 @@
         <v>47</v>
       </c>
       <c r="G187" s="18">
-        <v>2117</v>
+        <v>8795</v>
       </c>
       <c r="H187" s="21" t="s">
         <v>48</v>
@@ -8233,7 +8233,7 @@
         <v>47</v>
       </c>
       <c r="G188" s="13">
-        <v>3544</v>
+        <v>3135</v>
       </c>
       <c r="H188" s="17" t="s">
         <v>48</v>
@@ -8262,7 +8262,7 @@
         <v>47</v>
       </c>
       <c r="G189" s="18">
-        <v>2516</v>
+        <v>6640</v>
       </c>
       <c r="H189" s="21" t="s">
         <v>48</v>
@@ -8291,7 +8291,7 @@
         <v>47</v>
       </c>
       <c r="G190" s="13">
-        <v>5791</v>
+        <v>3089</v>
       </c>
       <c r="H190" s="17" t="s">
         <v>48</v>
@@ -8320,7 +8320,7 @@
         <v>47</v>
       </c>
       <c r="G191" s="18">
-        <v>5107</v>
+        <v>7709</v>
       </c>
       <c r="H191" s="21" t="s">
         <v>48</v>
@@ -8349,7 +8349,7 @@
         <v>436</v>
       </c>
       <c r="G192" s="13">
-        <v>7774</v>
+        <v>4876</v>
       </c>
       <c r="H192" s="17" t="s">
         <v>48</v>
@@ -8378,7 +8378,7 @@
         <v>436</v>
       </c>
       <c r="G193" s="18">
-        <v>2839</v>
+        <v>6894</v>
       </c>
       <c r="H193" s="21" t="s">
         <v>48</v>
@@ -8407,7 +8407,7 @@
         <v>436</v>
       </c>
       <c r="G194" s="13">
-        <v>4826</v>
+        <v>6545</v>
       </c>
       <c r="H194" s="17" t="s">
         <v>48</v>
@@ -8436,7 +8436,7 @@
         <v>436</v>
       </c>
       <c r="G195" s="18">
-        <v>4199</v>
+        <v>2700</v>
       </c>
       <c r="H195" s="21" t="s">
         <v>48</v>
@@ -8465,7 +8465,7 @@
         <v>436</v>
       </c>
       <c r="G196" s="13">
-        <v>1789</v>
+        <v>7629</v>
       </c>
       <c r="H196" s="17" t="s">
         <v>48</v>
@@ -8494,7 +8494,7 @@
         <v>436</v>
       </c>
       <c r="G197" s="18">
-        <v>2113</v>
+        <v>5294</v>
       </c>
       <c r="H197" s="21" t="s">
         <v>48</v>
@@ -8523,7 +8523,7 @@
         <v>436</v>
       </c>
       <c r="G198" s="13">
-        <v>5826</v>
+        <v>8852</v>
       </c>
       <c r="H198" s="17" t="s">
         <v>48</v>
@@ -8552,7 +8552,7 @@
         <v>436</v>
       </c>
       <c r="G199" s="18">
-        <v>2545</v>
+        <v>3467</v>
       </c>
       <c r="H199" s="21" t="s">
         <v>48</v>
@@ -8581,7 +8581,7 @@
         <v>436</v>
       </c>
       <c r="G200" s="13">
-        <v>4125</v>
+        <v>2191</v>
       </c>
       <c r="H200" s="17" t="s">
         <v>48</v>
@@ -8610,7 +8610,7 @@
         <v>436</v>
       </c>
       <c r="G201" s="18">
-        <v>7988</v>
+        <v>4139</v>
       </c>
       <c r="H201" s="21" t="s">
         <v>48</v>
@@ -8639,7 +8639,7 @@
         <v>436</v>
       </c>
       <c r="G202" s="13">
-        <v>2236</v>
+        <v>9144</v>
       </c>
       <c r="H202" s="17" t="s">
         <v>48</v>
@@ -8668,7 +8668,7 @@
         <v>436</v>
       </c>
       <c r="G203" s="18">
-        <v>4529</v>
+        <v>3784</v>
       </c>
       <c r="H203" s="21" t="s">
         <v>48</v>
@@ -8697,7 +8697,7 @@
         <v>436</v>
       </c>
       <c r="G204" s="13">
-        <v>4862</v>
+        <v>3324</v>
       </c>
       <c r="H204" s="17" t="s">
         <v>48</v>
@@ -8726,7 +8726,7 @@
         <v>436</v>
       </c>
       <c r="G205" s="18">
-        <v>7524</v>
+        <v>3444</v>
       </c>
       <c r="H205" s="21" t="s">
         <v>48</v>
@@ -8755,7 +8755,7 @@
         <v>436</v>
       </c>
       <c r="G206" s="13">
-        <v>4702</v>
+        <v>9087</v>
       </c>
       <c r="H206" s="17" t="s">
         <v>48</v>
@@ -8784,7 +8784,7 @@
         <v>436</v>
       </c>
       <c r="G207" s="18">
-        <v>4740</v>
+        <v>8684</v>
       </c>
       <c r="H207" s="21" t="s">
         <v>48</v>
@@ -8813,7 +8813,7 @@
         <v>436</v>
       </c>
       <c r="G208" s="13">
-        <v>3577</v>
+        <v>4069</v>
       </c>
       <c r="H208" s="17" t="s">
         <v>48</v>
@@ -8842,7 +8842,7 @@
         <v>436</v>
       </c>
       <c r="G209" s="18">
-        <v>2415</v>
+        <v>7460</v>
       </c>
       <c r="H209" s="21" t="s">
         <v>48</v>
@@ -8871,7 +8871,7 @@
         <v>436</v>
       </c>
       <c r="G210" s="13">
-        <v>8583</v>
+        <v>4842</v>
       </c>
       <c r="H210" s="17" t="s">
         <v>48</v>
@@ -8900,7 +8900,7 @@
         <v>436</v>
       </c>
       <c r="G211" s="18">
-        <v>2148</v>
+        <v>7390</v>
       </c>
       <c r="H211" s="21" t="s">
         <v>48</v>
@@ -8929,7 +8929,7 @@
         <v>436</v>
       </c>
       <c r="G212" s="13">
-        <v>5530</v>
+        <v>7363</v>
       </c>
       <c r="H212" s="17" t="s">
         <v>48</v>
@@ -8958,7 +8958,7 @@
         <v>436</v>
       </c>
       <c r="G213" s="18">
-        <v>5162</v>
+        <v>6814</v>
       </c>
       <c r="H213" s="21" t="s">
         <v>48</v>
@@ -8987,7 +8987,7 @@
         <v>436</v>
       </c>
       <c r="G214" s="13">
-        <v>3658</v>
+        <v>6846</v>
       </c>
       <c r="H214" s="17" t="s">
         <v>48</v>
@@ -9016,7 +9016,7 @@
         <v>436</v>
       </c>
       <c r="G215" s="18">
-        <v>2963</v>
+        <v>8397</v>
       </c>
       <c r="H215" s="21" t="s">
         <v>48</v>
@@ -9045,7 +9045,7 @@
         <v>436</v>
       </c>
       <c r="G216" s="13">
-        <v>5173</v>
+        <v>1977</v>
       </c>
       <c r="H216" s="17" t="s">
         <v>48</v>
@@ -9074,7 +9074,7 @@
         <v>436</v>
       </c>
       <c r="G217" s="18">
-        <v>7995</v>
+        <v>8636</v>
       </c>
       <c r="H217" s="21" t="s">
         <v>48</v>
@@ -9103,7 +9103,7 @@
         <v>436</v>
       </c>
       <c r="G218" s="13">
-        <v>4267</v>
+        <v>8915</v>
       </c>
       <c r="H218" s="17" t="s">
         <v>48</v>
@@ -9132,7 +9132,7 @@
         <v>436</v>
       </c>
       <c r="G219" s="18">
-        <v>2485</v>
+        <v>2339</v>
       </c>
       <c r="H219" s="21" t="s">
         <v>48</v>
@@ -9161,7 +9161,7 @@
         <v>436</v>
       </c>
       <c r="G220" s="13">
-        <v>4267</v>
+        <v>2242</v>
       </c>
       <c r="H220" s="17" t="s">
         <v>48</v>
@@ -9190,7 +9190,7 @@
         <v>436</v>
       </c>
       <c r="G221" s="18">
-        <v>6403</v>
+        <v>7033</v>
       </c>
       <c r="H221" s="21" t="s">
         <v>48</v>
@@ -9219,7 +9219,7 @@
         <v>436</v>
       </c>
       <c r="G222" s="13">
-        <v>7641</v>
+        <v>4659</v>
       </c>
       <c r="H222" s="17" t="s">
         <v>48</v>
@@ -9248,7 +9248,7 @@
         <v>436</v>
       </c>
       <c r="G223" s="18">
-        <v>4894</v>
+        <v>3199</v>
       </c>
       <c r="H223" s="21" t="s">
         <v>48</v>
@@ -9277,7 +9277,7 @@
         <v>436</v>
       </c>
       <c r="G224" s="13">
-        <v>4028</v>
+        <v>2246</v>
       </c>
       <c r="H224" s="17" t="s">
         <v>48</v>
@@ -9306,7 +9306,7 @@
         <v>436</v>
       </c>
       <c r="G225" s="18">
-        <v>1678</v>
+        <v>6173</v>
       </c>
       <c r="H225" s="21" t="s">
         <v>48</v>
@@ -9335,7 +9335,7 @@
         <v>436</v>
       </c>
       <c r="G226" s="13">
-        <v>4259</v>
+        <v>4226</v>
       </c>
       <c r="H226" s="17" t="s">
         <v>48</v>
@@ -9364,7 +9364,7 @@
         <v>436</v>
       </c>
       <c r="G227" s="18">
-        <v>1473</v>
+        <v>8069</v>
       </c>
       <c r="H227" s="21" t="s">
         <v>48</v>
@@ -9393,7 +9393,7 @@
         <v>436</v>
       </c>
       <c r="G228" s="13">
-        <v>3136</v>
+        <v>9075</v>
       </c>
       <c r="H228" s="17" t="s">
         <v>48</v>
@@ -9422,7 +9422,7 @@
         <v>436</v>
       </c>
       <c r="G229" s="18">
-        <v>7085</v>
+        <v>8252</v>
       </c>
       <c r="H229" s="21" t="s">
         <v>48</v>
@@ -9451,7 +9451,7 @@
         <v>436</v>
       </c>
       <c r="G230" s="13">
-        <v>8553</v>
+        <v>4486</v>
       </c>
       <c r="H230" s="17" t="s">
         <v>48</v>
@@ -9480,7 +9480,7 @@
         <v>436</v>
       </c>
       <c r="G231" s="18">
-        <v>8502</v>
+        <v>1663</v>
       </c>
       <c r="H231" s="21" t="s">
         <v>48</v>
@@ -9509,7 +9509,7 @@
         <v>47</v>
       </c>
       <c r="G232" s="13">
-        <v>9125</v>
+        <v>2715</v>
       </c>
       <c r="H232" s="17" t="s">
         <v>48</v>
@@ -9538,7 +9538,7 @@
         <v>47</v>
       </c>
       <c r="G233" s="18">
-        <v>4542</v>
+        <v>3605</v>
       </c>
       <c r="H233" s="21" t="s">
         <v>48</v>
@@ -9567,7 +9567,7 @@
         <v>47</v>
       </c>
       <c r="G234" s="13">
-        <v>2086</v>
+        <v>2302</v>
       </c>
       <c r="H234" s="17" t="s">
         <v>48</v>
@@ -9596,7 +9596,7 @@
         <v>47</v>
       </c>
       <c r="G235" s="18">
-        <v>5834</v>
+        <v>7554</v>
       </c>
       <c r="H235" s="21" t="s">
         <v>48</v>
@@ -9625,7 +9625,7 @@
         <v>47</v>
       </c>
       <c r="G236" s="13">
-        <v>5731</v>
+        <v>8531</v>
       </c>
       <c r="H236" s="17" t="s">
         <v>48</v>
@@ -9654,7 +9654,7 @@
         <v>47</v>
       </c>
       <c r="G237" s="18">
-        <v>8735</v>
+        <v>4360</v>
       </c>
       <c r="H237" s="21" t="s">
         <v>48</v>
@@ -9683,7 +9683,7 @@
         <v>47</v>
       </c>
       <c r="G238" s="13">
-        <v>7313</v>
+        <v>5442</v>
       </c>
       <c r="H238" s="17" t="s">
         <v>48</v>
@@ -9712,7 +9712,7 @@
         <v>47</v>
       </c>
       <c r="G239" s="18">
-        <v>4857</v>
+        <v>1986</v>
       </c>
       <c r="H239" s="21" t="s">
         <v>48</v>
@@ -9741,7 +9741,7 @@
         <v>47</v>
       </c>
       <c r="G240" s="13">
-        <v>6187</v>
+        <v>8353</v>
       </c>
       <c r="H240" s="17" t="s">
         <v>48</v>
@@ -9770,7 +9770,7 @@
         <v>47</v>
       </c>
       <c r="G241" s="18">
-        <v>4640</v>
+        <v>3933</v>
       </c>
       <c r="H241" s="21" t="s">
         <v>48</v>
@@ -9799,7 +9799,7 @@
         <v>47</v>
       </c>
       <c r="G242" s="13">
-        <v>6612</v>
+        <v>1414</v>
       </c>
       <c r="H242" s="17" t="s">
         <v>48</v>
@@ -9828,7 +9828,7 @@
         <v>47</v>
       </c>
       <c r="G243" s="18">
-        <v>5325</v>
+        <v>7062</v>
       </c>
       <c r="H243" s="21" t="s">
         <v>48</v>
@@ -9857,7 +9857,7 @@
         <v>47</v>
       </c>
       <c r="G244" s="13">
-        <v>3063</v>
+        <v>4414</v>
       </c>
       <c r="H244" s="17" t="s">
         <v>48</v>
@@ -9886,7 +9886,7 @@
         <v>47</v>
       </c>
       <c r="G245" s="18">
-        <v>5903</v>
+        <v>7682</v>
       </c>
       <c r="H245" s="21" t="s">
         <v>48</v>
@@ -9915,7 +9915,7 @@
         <v>47</v>
       </c>
       <c r="G246" s="13">
-        <v>2057</v>
+        <v>3369</v>
       </c>
       <c r="H246" s="17" t="s">
         <v>48</v>
@@ -9944,7 +9944,7 @@
         <v>47</v>
       </c>
       <c r="G247" s="18">
-        <v>2245</v>
+        <v>6513</v>
       </c>
       <c r="H247" s="21" t="s">
         <v>48</v>
@@ -9973,7 +9973,7 @@
         <v>47</v>
       </c>
       <c r="G248" s="13">
-        <v>8644</v>
+        <v>7405</v>
       </c>
       <c r="H248" s="17" t="s">
         <v>48</v>
@@ -10002,7 +10002,7 @@
         <v>47</v>
       </c>
       <c r="G249" s="18">
-        <v>2591</v>
+        <v>4771</v>
       </c>
       <c r="H249" s="21" t="s">
         <v>48</v>
@@ -10031,7 +10031,7 @@
         <v>47</v>
       </c>
       <c r="G250" s="13">
-        <v>7022</v>
+        <v>3605</v>
       </c>
       <c r="H250" s="17" t="s">
         <v>48</v>
@@ -10060,7 +10060,7 @@
         <v>47</v>
       </c>
       <c r="G251" s="18">
-        <v>1234</v>
+        <v>2573</v>
       </c>
       <c r="H251" s="21" t="s">
         <v>48</v>
@@ -10089,7 +10089,7 @@
         <v>47</v>
       </c>
       <c r="G252" s="13">
-        <v>2330</v>
+        <v>4829</v>
       </c>
       <c r="H252" s="17" t="s">
         <v>48</v>
@@ -10118,7 +10118,7 @@
         <v>47</v>
       </c>
       <c r="G253" s="18">
-        <v>2608</v>
+        <v>5763</v>
       </c>
       <c r="H253" s="21" t="s">
         <v>48</v>
@@ -10147,7 +10147,7 @@
         <v>47</v>
       </c>
       <c r="G254" s="13">
-        <v>4718</v>
+        <v>4204</v>
       </c>
       <c r="H254" s="17" t="s">
         <v>48</v>
@@ -10176,7 +10176,7 @@
         <v>47</v>
       </c>
       <c r="G255" s="18">
-        <v>7803</v>
+        <v>2800</v>
       </c>
       <c r="H255" s="21" t="s">
         <v>48</v>
@@ -10205,7 +10205,7 @@
         <v>47</v>
       </c>
       <c r="G256" s="13">
-        <v>7607</v>
+        <v>8475</v>
       </c>
       <c r="H256" s="17" t="s">
         <v>48</v>
@@ -10234,7 +10234,7 @@
         <v>47</v>
       </c>
       <c r="G257" s="18">
-        <v>4666</v>
+        <v>4713</v>
       </c>
       <c r="H257" s="21" t="s">
         <v>48</v>
@@ -10263,7 +10263,7 @@
         <v>47</v>
       </c>
       <c r="G258" s="13">
-        <v>2688</v>
+        <v>1727</v>
       </c>
       <c r="H258" s="17" t="s">
         <v>48</v>
@@ -10292,7 +10292,7 @@
         <v>47</v>
       </c>
       <c r="G259" s="18">
-        <v>2042</v>
+        <v>8648</v>
       </c>
       <c r="H259" s="21" t="s">
         <v>48</v>
@@ -10321,7 +10321,7 @@
         <v>47</v>
       </c>
       <c r="G260" s="13">
-        <v>2384</v>
+        <v>4695</v>
       </c>
       <c r="H260" s="17" t="s">
         <v>48</v>
@@ -10350,7 +10350,7 @@
         <v>47</v>
       </c>
       <c r="G261" s="18">
-        <v>2568</v>
+        <v>4179</v>
       </c>
       <c r="H261" s="21" t="s">
         <v>48</v>
@@ -10379,7 +10379,7 @@
         <v>47</v>
       </c>
       <c r="G262" s="13">
-        <v>7177</v>
+        <v>6127</v>
       </c>
       <c r="H262" s="17" t="s">
         <v>48</v>
@@ -10408,7 +10408,7 @@
         <v>47</v>
       </c>
       <c r="G263" s="18">
-        <v>3181</v>
+        <v>8443</v>
       </c>
       <c r="H263" s="21" t="s">
         <v>48</v>
@@ -10437,7 +10437,7 @@
         <v>47</v>
       </c>
       <c r="G264" s="13">
-        <v>5937</v>
+        <v>5097</v>
       </c>
       <c r="H264" s="17" t="s">
         <v>48</v>
@@ -10466,7 +10466,7 @@
         <v>47</v>
       </c>
       <c r="G265" s="18">
-        <v>7382</v>
+        <v>1940</v>
       </c>
       <c r="H265" s="21" t="s">
         <v>48</v>
@@ -10495,7 +10495,7 @@
         <v>47</v>
       </c>
       <c r="G266" s="13">
-        <v>4142</v>
+        <v>1399</v>
       </c>
       <c r="H266" s="17" t="s">
         <v>48</v>
@@ -10524,7 +10524,7 @@
         <v>47</v>
       </c>
       <c r="G267" s="18">
-        <v>6227</v>
+        <v>6493</v>
       </c>
       <c r="H267" s="21" t="s">
         <v>48</v>
@@ -10553,7 +10553,7 @@
         <v>47</v>
       </c>
       <c r="G268" s="13">
-        <v>2726</v>
+        <v>1201</v>
       </c>
       <c r="H268" s="17" t="s">
         <v>48</v>
@@ -10582,7 +10582,7 @@
         <v>47</v>
       </c>
       <c r="G269" s="18">
-        <v>7692</v>
+        <v>2865</v>
       </c>
       <c r="H269" s="21" t="s">
         <v>48</v>
@@ -10611,7 +10611,7 @@
         <v>47</v>
       </c>
       <c r="G270" s="13">
-        <v>6105</v>
+        <v>2443</v>
       </c>
       <c r="H270" s="17" t="s">
         <v>48</v>
@@ -10640,7 +10640,7 @@
         <v>47</v>
       </c>
       <c r="G271" s="18">
-        <v>3584</v>
+        <v>7261</v>
       </c>
       <c r="H271" s="21" t="s">
         <v>48</v>
@@ -10669,7 +10669,7 @@
         <v>47</v>
       </c>
       <c r="G272" s="13">
-        <v>6855</v>
+        <v>5706</v>
       </c>
       <c r="H272" s="17" t="s">
         <v>48</v>
@@ -10698,7 +10698,7 @@
         <v>47</v>
       </c>
       <c r="G273" s="18">
-        <v>2944</v>
+        <v>6336</v>
       </c>
       <c r="H273" s="21" t="s">
         <v>48</v>
@@ -10727,7 +10727,7 @@
         <v>47</v>
       </c>
       <c r="G274" s="13">
-        <v>2501</v>
+        <v>7427</v>
       </c>
       <c r="H274" s="17" t="s">
         <v>48</v>
@@ -10756,7 +10756,7 @@
         <v>47</v>
       </c>
       <c r="G275" s="18">
-        <v>3566</v>
+        <v>3255</v>
       </c>
       <c r="H275" s="21" t="s">
         <v>48</v>
@@ -10785,7 +10785,7 @@
         <v>47</v>
       </c>
       <c r="G276" s="13">
-        <v>8176</v>
+        <v>4793</v>
       </c>
       <c r="H276" s="17" t="s">
         <v>48</v>
@@ -10814,7 +10814,7 @@
         <v>47</v>
       </c>
       <c r="G277" s="18">
-        <v>3897</v>
+        <v>8338</v>
       </c>
       <c r="H277" s="21" t="s">
         <v>48</v>
@@ -10843,7 +10843,7 @@
         <v>47</v>
       </c>
       <c r="G278" s="13">
-        <v>4426</v>
+        <v>1442</v>
       </c>
       <c r="H278" s="17" t="s">
         <v>48</v>
@@ -10872,7 +10872,7 @@
         <v>47</v>
       </c>
       <c r="G279" s="18">
-        <v>4142</v>
+        <v>4894</v>
       </c>
       <c r="H279" s="21" t="s">
         <v>48</v>
@@ -10901,7 +10901,7 @@
         <v>47</v>
       </c>
       <c r="G280" s="13">
-        <v>1214</v>
+        <v>6938</v>
       </c>
       <c r="H280" s="17" t="s">
         <v>48</v>
@@ -10930,7 +10930,7 @@
         <v>47</v>
       </c>
       <c r="G281" s="18">
-        <v>3696</v>
+        <v>3445</v>
       </c>
       <c r="H281" s="21" t="s">
         <v>48</v>
@@ -10959,7 +10959,7 @@
         <v>47</v>
       </c>
       <c r="G282" s="13">
-        <v>2614</v>
+        <v>6350</v>
       </c>
       <c r="H282" s="17" t="s">
         <v>48</v>
@@ -10988,7 +10988,7 @@
         <v>47</v>
       </c>
       <c r="G283" s="18">
-        <v>5278</v>
+        <v>2310</v>
       </c>
       <c r="H283" s="21" t="s">
         <v>48</v>
@@ -11017,7 +11017,7 @@
         <v>47</v>
       </c>
       <c r="G284" s="13">
-        <v>5809</v>
+        <v>2071</v>
       </c>
       <c r="H284" s="17" t="s">
         <v>48</v>
@@ -11046,7 +11046,7 @@
         <v>47</v>
       </c>
       <c r="G285" s="18">
-        <v>2512</v>
+        <v>7012</v>
       </c>
       <c r="H285" s="21" t="s">
         <v>48</v>
@@ -11075,7 +11075,7 @@
         <v>47</v>
       </c>
       <c r="G286" s="13">
-        <v>7447</v>
+        <v>6716</v>
       </c>
       <c r="H286" s="17" t="s">
         <v>48</v>
@@ -11104,7 +11104,7 @@
         <v>47</v>
       </c>
       <c r="G287" s="18">
-        <v>3953</v>
+        <v>3535</v>
       </c>
       <c r="H287" s="21" t="s">
         <v>48</v>
@@ -11133,7 +11133,7 @@
         <v>47</v>
       </c>
       <c r="G288" s="13">
-        <v>1866</v>
+        <v>5011</v>
       </c>
       <c r="H288" s="17" t="s">
         <v>48</v>
@@ -11162,7 +11162,7 @@
         <v>47</v>
       </c>
       <c r="G289" s="18">
-        <v>1917</v>
+        <v>5630</v>
       </c>
       <c r="H289" s="21" t="s">
         <v>48</v>
@@ -11191,7 +11191,7 @@
         <v>47</v>
       </c>
       <c r="G290" s="13">
-        <v>5391</v>
+        <v>7442</v>
       </c>
       <c r="H290" s="17" t="s">
         <v>48</v>
@@ -11220,7 +11220,7 @@
         <v>47</v>
       </c>
       <c r="G291" s="18">
-        <v>1980</v>
+        <v>4064</v>
       </c>
       <c r="H291" s="21" t="s">
         <v>48</v>
@@ -11249,7 +11249,7 @@
         <v>47</v>
       </c>
       <c r="G292" s="13">
-        <v>4860</v>
+        <v>6924</v>
       </c>
       <c r="H292" s="17" t="s">
         <v>48</v>
@@ -11278,7 +11278,7 @@
         <v>47</v>
       </c>
       <c r="G293" s="18">
-        <v>3568</v>
+        <v>2978</v>
       </c>
       <c r="H293" s="21" t="s">
         <v>48</v>
@@ -11307,7 +11307,7 @@
         <v>47</v>
       </c>
       <c r="G294" s="13">
-        <v>6949</v>
+        <v>5811</v>
       </c>
       <c r="H294" s="17" t="s">
         <v>48</v>
@@ -11336,7 +11336,7 @@
         <v>47</v>
       </c>
       <c r="G295" s="18">
-        <v>2410</v>
+        <v>3183</v>
       </c>
       <c r="H295" s="21" t="s">
         <v>48</v>
@@ -11365,7 +11365,7 @@
         <v>47</v>
       </c>
       <c r="G296" s="13">
-        <v>5857</v>
+        <v>1476</v>
       </c>
       <c r="H296" s="17" t="s">
         <v>48</v>
@@ -11394,7 +11394,7 @@
         <v>47</v>
       </c>
       <c r="G297" s="18">
-        <v>3984</v>
+        <v>3672</v>
       </c>
       <c r="H297" s="21" t="s">
         <v>48</v>
@@ -11423,7 +11423,7 @@
         <v>47</v>
       </c>
       <c r="G298" s="13">
-        <v>1917</v>
+        <v>4315</v>
       </c>
       <c r="H298" s="17" t="s">
         <v>48</v>
@@ -11452,7 +11452,7 @@
         <v>47</v>
       </c>
       <c r="G299" s="18">
-        <v>1881</v>
+        <v>7562</v>
       </c>
       <c r="H299" s="21" t="s">
         <v>48</v>
@@ -11481,7 +11481,7 @@
         <v>47</v>
       </c>
       <c r="G300" s="13">
-        <v>3494</v>
+        <v>1555</v>
       </c>
       <c r="H300" s="17" t="s">
         <v>48</v>
@@ -11510,7 +11510,7 @@
         <v>47</v>
       </c>
       <c r="G301" s="18">
-        <v>4067</v>
+        <v>7485</v>
       </c>
       <c r="H301" s="21" t="s">
         <v>48</v>

</xml_diff>